<commit_message>
Excel: remove all green backgrounds + add References and Glossary tabs
- All table headers: green #2B5A18 → charcoal #2D2D2D
- All light green fills (F0F7EC, E4FCC0): replaced with neutral grays
- New tab: References — 11 sources with clickable URLs and confidence ratings
- New tab: Glossary — 27 terms (POD, Decorator, MAT-001, FTC, kill gate, schema fields...)
- Output path updated to deliverables/

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/FYUL_Leather_Financial_Model.xlsx
+++ b/deliverables/FYUL_Leather_Financial_Model.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Benchmark" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -146,7 +148,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -160,7 +162,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002B5A18"/>
+        <fgColor rgb="002D2D2D"/>
       </patternFill>
     </fill>
     <fill>
@@ -170,17 +172,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4FCC0"/>
+        <fgColor rgb="00EBEBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAF6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0F7EC"/>
       </patternFill>
     </fill>
     <fill>
@@ -284,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -393,202 +390,172 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -600,16 +567,22 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2855,17 +2828,17 @@
           <t>1 · Low-Friction Onboarding</t>
         </is>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>KR 1.1</t>
         </is>
       </c>
-      <c r="C6" s="40" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Decorator onboarding time (portal → first approved blueprint)</t>
         </is>
       </c>
-      <c r="D6" s="41" t="inlineStr">
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>No leather portal today. Generic multi-field form without AI assist = 3–5 days (email back-and-forth)</t>
         </is>
@@ -2875,22 +2848,22 @@
           <t>&lt; 24 hours</t>
         </is>
       </c>
-      <c r="F6" s="40" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Each day of delay = supply bottleneck. Long onboarding → Decorator abandonment → 150-SKU pilot fails before launch</t>
         </is>
       </c>
-      <c r="G6" s="42" t="inlineStr">
+      <c r="G6" s="40" t="inlineStr">
         <is>
           <t>Printify apparel onboarding benchmark: complex forms without AI assist average 3–5 days. AI field-assist pre-fills 8 schema fields → estimated 70% reduction. Target 24h is achievable with assisted flow.</t>
         </is>
       </c>
-      <c r="H6" s="43" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>MVP 2</t>
         </is>
       </c>
-      <c r="I6" s="43" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>⚪ Not started</t>
         </is>
@@ -2902,17 +2875,17 @@
           <t>1 · Low-Friction Onboarding</t>
         </is>
       </c>
-      <c r="B7" s="39" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>KR 1.2</t>
         </is>
       </c>
-      <c r="C7" s="40" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Portal submission form error rate (rejected / total submitted)</t>
         </is>
       </c>
-      <c r="D7" s="41" t="inlineStr">
+      <c r="D7" s="39" t="inlineStr">
         <is>
           <t>Estimated 20–35% error rate on unassisted complex multi-field material forms (industry benchmark)</t>
         </is>
@@ -2922,34 +2895,34 @@
           <t>&lt; 10%</t>
         </is>
       </c>
-      <c r="F7" s="40" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>&gt;20% error rate → manual Ops queue required. Each manual review costs ~$40 ops vs. $8 margin/order — unit economics collapse at any volume above pilot</t>
         </is>
       </c>
-      <c r="G7" s="42" t="inlineStr">
+      <c r="G7" s="40" t="inlineStr">
         <is>
           <t>Industry benchmark: unassisted 5+ field enum forms average 20–35% error rate. Field-Assist Agent (AI pre-fill) reduces error rate to &lt;10% in comparable deployments (Printify internal UX data).</t>
         </is>
       </c>
-      <c r="H7" s="43" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>MVP 2 Gate</t>
         </is>
       </c>
-      <c r="I7" s="43" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>⚪ Not started</t>
         </is>
       </c>
     </row>
     <row r="8" ht="56" customHeight="1">
-      <c r="A8" s="44" t="inlineStr">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>2 · Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="B8" s="45" t="inlineStr">
+      <c r="B8" s="42" t="inlineStr">
         <is>
           <t>KR 2.1</t>
         </is>
@@ -2959,7 +2932,7 @@
           <t>MAT-001 FTC classifier auto-approval rate (genuine leather submissions)</t>
         </is>
       </c>
-      <c r="D8" s="46" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>0% auto-approval. No classifier today — 100% of leather submissions require manual compliance review</t>
         </is>
@@ -2974,7 +2947,7 @@
           <t>&lt;88% auto-approval = manual ops scale linearly with volume. At 3,000 orders/mo, manual review destroys the $8 margin/order. 88% sets a floor where ops queue remains manageable</t>
         </is>
       </c>
-      <c r="G8" s="47" t="inlineStr">
+      <c r="G8" s="44" t="inlineStr">
         <is>
           <t>LLM classifiers on structured-label material tasks achieve 85–92% accuracy (Printify compliance team estimate). 88% is the break-even point where automated review covers &gt;10 Decorator catalog scale without additional ops headcount.</t>
         </is>
@@ -2991,12 +2964,12 @@
       </c>
     </row>
     <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="44" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>2 · Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="B9" s="45" t="inlineStr">
+      <c r="B9" s="42" t="inlineStr">
         <is>
           <t>KR 2.2</t>
         </is>
@@ -3006,7 +2979,7 @@
           <t>FTC MAT-001 false-positive rate (legitimate Decorators wrongly rejected)</t>
         </is>
       </c>
-      <c r="D9" s="46" t="inlineStr">
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>N/A today — no classifier. PU/bonded leather is listed as "genuine" with zero enforcement</t>
         </is>
@@ -3021,7 +2994,7 @@
           <t>FP &gt; 2% = legitimate Decorators wrongly blocked → churned account + platform trust damage. Every false block is a supply loss and a reputational risk.</t>
         </is>
       </c>
-      <c r="G9" s="47" t="inlineStr">
+      <c r="G9" s="44" t="inlineStr">
         <is>
           <t>Internal Printify UX benchmark: &lt;2% false rejection rate is the acceptable threshold for gated submission flows. Above 2%, user trust collapses and appeal volume overwhelms Ops (Printify apparel classifier precedent).</t>
         </is>
@@ -3043,17 +3016,17 @@
           <t>3 · Commercial ROI &amp; Velocity</t>
         </is>
       </c>
-      <c r="B10" s="39" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>KR 3.1</t>
         </is>
       </c>
-      <c r="C10" s="40" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Active catalog SKUs live before marketplace launch (Etsy + Amazon + Shopify)</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>0 genuine leather SKUs on Printify today (confirmed: internal catalog audit — 45 products, 100% synthetic PU)</t>
         </is>
@@ -3063,22 +3036,22 @@
           <t>150 SKUs (5×30)</t>
         </is>
       </c>
-      <c r="F10" s="40" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Etsy and Amazon algorithms require minimum catalog depth to surface a new supplier organically. Below 100 active listings = category-invisible. Shopify pilot (W12) starts earlier with fewer SKUs and provides immediate signal.</t>
         </is>
       </c>
-      <c r="G10" s="42" t="inlineStr">
+      <c r="G10" s="40" t="inlineStr">
         <is>
           <t>eRank: minimum ~100 active listings required for category algorithm indexing signal. ShelfTrend: top-quartile leather stores average 120–200 active SKUs. Shopify Material Attributes (2025): no indexing delay — W12 signal valid from day 1.</t>
         </is>
       </c>
-      <c r="H10" s="43" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>MVP 2 Gate</t>
         </is>
       </c>
-      <c r="I10" s="43" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>⚪ Not started</t>
         </is>
@@ -3090,17 +3063,17 @@
           <t>3 · Commercial ROI &amp; Velocity</t>
         </is>
       </c>
-      <c r="B11" s="39" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>KR 3.2</t>
         </is>
       </c>
-      <c r="C11" s="40" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Sales velocity post-launch: orders / SKU / month (organic, all channels)</t>
         </is>
       </c>
-      <c r="D11" s="41" t="inlineStr">
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>0 orders/SKU/mo on Printify leather (no genuine leather exists today)</t>
         </is>
@@ -3110,22 +3083,22 @@
           <t>≥ 20 / SKU / mo</t>
         </is>
       </c>
-      <c r="F11" s="40" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>20/SKU is the base-case planning floor for positive ROI on $340K investment (payback ~16 months). Kill gate triggers at &lt;15 at Month 2 — 20 gives a 33% safety margin above the kill threshold.</t>
         </is>
       </c>
-      <c r="G11" s="42" t="inlineStr">
+      <c r="G11" s="40" t="inlineStr">
         <is>
           <t>Proxy: accio.com — BULLIANT leather wallet (Amazon) = 8,365 units/mo. Etsy top-quartile leather sellers: 15–25 orders/SKU/mo (ShelfTrend 2025). 20/SKU is achievable entry point within documented range. Shopify adds a 3rd channel reducing single-platform dependency.</t>
         </is>
       </c>
-      <c r="H11" s="43" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>MVP 3 / Month 1</t>
         </is>
       </c>
-      <c r="I11" s="43" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>⚪ Not started</t>
         </is>
@@ -3137,17 +3110,17 @@
           <t>3 · Commercial ROI &amp; Velocity</t>
         </is>
       </c>
-      <c r="B12" s="39" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>KR 3.3</t>
         </is>
       </c>
-      <c r="C12" s="40" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>Monthly Printify platform margin (leather category, post-pilot scale)</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="39" t="inlineStr">
         <is>
           <t>$0/month leather platform margin (no genuine leather GMV on Printify today)</t>
         </is>
@@ -3157,22 +3130,22 @@
           <t>$150K / month</t>
         </is>
       </c>
-      <c r="F12" s="40" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>$340K investment requires ~$150K/mo run-rate to achieve the ~16-month payback (base case). Below $60K/mo at Month 3 = ROI thesis fails and investment is not recovered on schedule.</t>
         </is>
       </c>
-      <c r="G12" s="42" t="inlineStr">
+      <c r="G12" s="40" t="inlineStr">
         <is>
           <t>10 Dec × 150 SKUs × 20 orders × $8 margin = $150K/mo target. Etsy category GMV proxy: $130K–$270K/week leather category (ShelfTrend 2025) supports 20/SKU base case. Shopify (MVP 2) adds incremental demand channel improving base-case achievability.</t>
         </is>
       </c>
-      <c r="H12" s="43" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="I12" s="43" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>⚪ Not started</t>
         </is>
@@ -3231,7 +3204,7 @@
           <t>Orders / SKU / month</t>
         </is>
       </c>
-      <c r="B17" s="48" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>0 (no genuine leather today)</t>
         </is>
@@ -3241,17 +3214,17 @@
           <t>≥ 20 (base) · ≥ 50 (opt)</t>
         </is>
       </c>
-      <c r="D17" s="49" t="inlineStr">
+      <c r="D17" s="45" t="inlineStr">
         <is>
           <t>≥ 20 sustained</t>
         </is>
       </c>
-      <c r="E17" s="50" t="inlineStr">
+      <c r="E17" s="46" t="inlineStr">
         <is>
           <t>&lt; 15 at Month 2 → KILL</t>
         </is>
       </c>
-      <c r="F17" s="51" t="inlineStr">
+      <c r="F17" s="40" t="inlineStr">
         <is>
           <t>Platform order data · leather material_tier tag</t>
         </is>
@@ -3268,7 +3241,7 @@
           <t>FTC MAT-001 auto-approve %</t>
         </is>
       </c>
-      <c r="B18" s="46" t="inlineStr">
+      <c r="B18" s="43" t="inlineStr">
         <is>
           <t>0% (100% manual review today)</t>
         </is>
@@ -3283,12 +3256,12 @@
           <t>≥ 88%</t>
         </is>
       </c>
-      <c r="E18" s="52" t="inlineStr">
+      <c r="E18" s="47" t="inlineStr">
         <is>
           <t>FP rate &gt; 2% → PAUSE MVP 1</t>
         </is>
       </c>
-      <c r="F18" s="47" t="inlineStr">
+      <c r="F18" s="44" t="inlineStr">
         <is>
           <t>Ingestion logs · MAT-001 classifier output</t>
         </is>
@@ -3305,7 +3278,7 @@
           <t>Decorator form error rate</t>
         </is>
       </c>
-      <c r="B19" s="48" t="inlineStr">
+      <c r="B19" s="39" t="inlineStr">
         <is>
           <t>~20–35% (industry benchmark, no AI assist)</t>
         </is>
@@ -3315,7 +3288,7 @@
           <t>&lt; 10%</t>
         </is>
       </c>
-      <c r="D19" s="49" t="inlineStr">
+      <c r="D19" s="45" t="inlineStr">
         <is>
           <t>&lt; 10%</t>
         </is>
@@ -3325,7 +3298,7 @@
           <t>&gt; 20% → redesign portal + AI flow</t>
         </is>
       </c>
-      <c r="F19" s="51" t="inlineStr">
+      <c r="F19" s="40" t="inlineStr">
         <is>
           <t>Portal submission logs (rejected / total)</t>
         </is>
@@ -3342,7 +3315,7 @@
           <t>Decorator onboarding time</t>
         </is>
       </c>
-      <c r="B20" s="46" t="inlineStr">
+      <c r="B20" s="43" t="inlineStr">
         <is>
           <t>No leather portal · est. 3–5 days via email</t>
         </is>
@@ -3362,7 +3335,7 @@
           <t>&gt; 48h avg → UX rework</t>
         </is>
       </c>
-      <c r="F20" s="47" t="inlineStr">
+      <c r="F20" s="44" t="inlineStr">
         <is>
           <t>Portal timestamp (form start → first approved blueprint)</t>
         </is>
@@ -3379,7 +3352,7 @@
           <t>Monthly platform margin</t>
         </is>
       </c>
-      <c r="B21" s="48" t="inlineStr">
+      <c r="B21" s="39" t="inlineStr">
         <is>
           <t>$0 (no leather GMV today)</t>
         </is>
@@ -3389,7 +3362,7 @@
           <t>$24K (pilot: 150 SKUs base case)</t>
         </is>
       </c>
-      <c r="D21" s="49" t="inlineStr">
+      <c r="D21" s="45" t="inlineStr">
         <is>
           <t>$150K (base) / $375K (opt)</t>
         </is>
@@ -3399,7 +3372,7 @@
           <t>&lt; $10K at Month 3 → re-evaluate ROI</t>
         </is>
       </c>
-      <c r="F21" s="51" t="inlineStr">
+      <c r="F21" s="40" t="inlineStr">
         <is>
           <t>GMV dashboard · leather category tag</t>
         </is>
@@ -3416,7 +3389,7 @@
           <t>Active catalog SKUs</t>
         </is>
       </c>
-      <c r="B22" s="46" t="inlineStr">
+      <c r="B22" s="43" t="inlineStr">
         <is>
           <t>0 genuine leather SKUs (catalog audit confirmed)</t>
         </is>
@@ -3436,7 +3409,7 @@
           <t>&lt; 100 at MVP 2 Gate → delay launch</t>
         </is>
       </c>
-      <c r="F22" s="47" t="inlineStr">
+      <c r="F22" s="44" t="inlineStr">
         <is>
           <t>Blueprint DB · material_tier ≠ null</t>
         </is>
@@ -3453,7 +3426,7 @@
           <t>Merchant listing rate</t>
         </is>
       </c>
-      <c r="B23" s="48" t="inlineStr">
+      <c r="B23" s="39" t="inlineStr">
         <is>
           <t>N/A (no leather portal or supply path today)</t>
         </is>
@@ -3463,7 +3436,7 @@
           <t>≥ 60% of enrolled Decorators</t>
         </is>
       </c>
-      <c r="D23" s="49" t="inlineStr">
+      <c r="D23" s="45" t="inlineStr">
         <is>
           <t>≥ 70%</t>
         </is>
@@ -3473,7 +3446,7 @@
           <t>&lt; 40% → supply conversion problem</t>
         </is>
       </c>
-      <c r="F23" s="51" t="inlineStr">
+      <c r="F23" s="40" t="inlineStr">
         <is>
           <t>Enrolled Decorators → active listings ratio</t>
         </is>
@@ -3490,7 +3463,7 @@
           <t>Platform margin / order</t>
         </is>
       </c>
-      <c r="B24" s="46" t="inlineStr">
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>$5/order (apparel average on Printify)</t>
         </is>
@@ -3510,7 +3483,7 @@
           <t>Below $6 → renegotiate supplier pricing</t>
         </is>
       </c>
-      <c r="F24" s="47" t="inlineStr">
+      <c r="F24" s="44" t="inlineStr">
         <is>
           <t>Order margin report · leather category filter</t>
         </is>
@@ -3582,12 +3555,12 @@
           <t>≥ 5 Signed Decorator LOIs + Supplier SLA confirmed</t>
         </is>
       </c>
-      <c r="D29" s="53" t="inlineStr">
+      <c r="D29" s="48" t="inlineStr">
         <is>
           <t>Approve ~$20K Design Sprint</t>
         </is>
       </c>
-      <c r="E29" s="54" t="inlineStr">
+      <c r="E29" s="49" t="inlineStr">
         <is>
           <t>CANCEL — $0 engineering spent</t>
         </is>
@@ -3619,12 +3592,12 @@
           <t>150 valid leather SKUs created · portal error rate &lt; 10%</t>
         </is>
       </c>
-      <c r="D30" s="55" t="inlineStr">
+      <c r="D30" s="50" t="inlineStr">
         <is>
           <t>Proceed to Marketplace build</t>
         </is>
       </c>
-      <c r="E30" s="52" t="inlineStr">
+      <c r="E30" s="47" t="inlineStr">
         <is>
           <t>PAUSE — redesign portal UI + AI field-assist flow</t>
         </is>
@@ -3641,37 +3614,37 @@
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="56" t="inlineStr">
+      <c r="A31" s="51" t="inlineStr">
         <is>
           <t>Gate 2 · M2</t>
         </is>
       </c>
-      <c r="B31" s="57" t="inlineStr">
+      <c r="B31" s="52" t="inlineStr">
         <is>
           <t>Month 2 post-M0</t>
         </is>
       </c>
-      <c r="C31" s="57" t="inlineStr">
+      <c r="C31" s="52" t="inlineStr">
         <is>
           <t>≥ 20 orders / SKU / month (organic, all channels)</t>
         </is>
       </c>
-      <c r="D31" s="58" t="inlineStr">
+      <c r="D31" s="53" t="inlineStr">
         <is>
           <t>FULL SCALE to 1,500+ SKUs</t>
         </is>
       </c>
-      <c r="E31" s="50" t="inlineStr">
+      <c r="E31" s="46" t="inlineStr">
         <is>
           <t>KILL (&lt; 15) — halt &amp; reallocate team</t>
         </is>
       </c>
-      <c r="F31" s="57" t="inlineStr">
+      <c r="F31" s="52" t="inlineStr">
         <is>
           <t>~$340K</t>
         </is>
       </c>
-      <c r="G31" s="57" t="inlineStr">
+      <c r="G31" s="52" t="inlineStr">
         <is>
           <t>Shopify: immediate signal from W12. Etsy/Amazon: 30-day indexing delay → M2 is first clean read. M1 = launch noise.</t>
         </is>
@@ -3834,7 +3807,7 @@
           <t>#215 top search term · $35–$70 AOV · 125%+ CTR</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="54" t="inlineStr">
         <is>
           <t>ShelfTrend 2025</t>
         </is>
@@ -3866,7 +3839,7 @@
           <t>$130K–$270K / week</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="55" t="inlineStr">
         <is>
           <t>ShelfTrend 2025</t>
         </is>
@@ -3898,7 +3871,7 @@
           <t>BULLIANT wallet — 8,365 units / month (BSR rank)</t>
         </is>
       </c>
-      <c r="D7" s="59" t="inlineStr">
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>accio.com 2025</t>
         </is>
@@ -3930,12 +3903,12 @@
           <t>$54.26B total · 6.7% CAGR · custom/POD ~$2B addressable (est.)</t>
         </is>
       </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="D8" s="55" t="inlineStr">
         <is>
           <t>Nova One Advisor 2025</t>
         </is>
       </c>
-      <c r="E8" s="52" t="inlineStr">
+      <c r="E8" s="47" t="inlineStr">
         <is>
           <t>Low–Medium</t>
         </is>
@@ -4026,7 +3999,7 @@
           <t>#215 top keyword · +57% search volume growth Nov–Dec (gifting peak)</t>
         </is>
       </c>
-      <c r="D11" s="59" t="inlineStr">
+      <c r="D11" s="54" t="inlineStr">
         <is>
           <t>eRank 2025</t>
         </is>
@@ -4058,7 +4031,7 @@
           <t>50-unit minimum order · no taxonomy fields · no FTC compliance</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr">
+      <c r="D12" s="55" t="inlineStr">
         <is>
           <t>Public pricing (printKK.com)</t>
         </is>
@@ -4095,7 +4068,7 @@
           <t>PM hypothesis</t>
         </is>
       </c>
-      <c r="E13" s="54" t="inlineStr">
+      <c r="E13" s="49" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -4145,7 +4118,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C18" s="56" t="inlineStr">
         <is>
           <t>PoC outreach: 50 existing Printify customers → ~10% conversion → ≥ 5 LOIs</t>
         </is>
@@ -4160,12 +4133,12 @@
           <t>SKUs per Decorator</t>
         </is>
       </c>
-      <c r="B19" s="62" t="inlineStr">
+      <c r="B19" s="57" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="C19" s="63" t="inlineStr">
+      <c r="C19" s="58" t="inlineStr">
         <is>
           <t>Each Decorator lists 30 products (wallets, bags, journals, belts)</t>
         </is>
@@ -4185,7 +4158,7 @@
           <t>150</t>
         </is>
       </c>
-      <c r="C20" s="61" t="inlineStr">
+      <c r="C20" s="56" t="inlineStr">
         <is>
           <t>5 × 30 = 150 · minimum for marketplace algorithm indexing</t>
         </is>
@@ -4205,7 +4178,7 @@
           <t>$8</t>
         </is>
       </c>
-      <c r="C21" s="63" t="inlineStr">
+      <c r="C21" s="58" t="inlineStr">
         <is>
           <t>Premium leather AOV $45–65 supports $8 vs. standard $5 for apparel</t>
         </is>
@@ -4225,7 +4198,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C22" s="61" t="inlineStr">
+      <c r="C22" s="56" t="inlineStr">
         <is>
           <t>Top-quartile Etsy leather sellers proxy (kill threshold = &lt; 15 at Month 2)</t>
         </is>
@@ -4240,12 +4213,12 @@
           <t>Monthly orders (pilot)</t>
         </is>
       </c>
-      <c r="B23" s="62" t="inlineStr">
+      <c r="B23" s="57" t="inlineStr">
         <is>
           <t>3,000</t>
         </is>
       </c>
-      <c r="C23" s="63" t="inlineStr">
+      <c r="C23" s="58" t="inlineStr">
         <is>
           <t>150 SKUs × 20 orders = 3,000 orders/month</t>
         </is>
@@ -4265,7 +4238,7 @@
           <t>$24,000</t>
         </is>
       </c>
-      <c r="C24" s="61" t="inlineStr">
+      <c r="C24" s="56" t="inlineStr">
         <is>
           <t>3,000 orders × $8 = $24K/month during pilot phase</t>
         </is>
@@ -4285,7 +4258,7 @@
           <t>$150,000</t>
         </is>
       </c>
-      <c r="C25" s="63" t="inlineStr">
+      <c r="C25" s="58" t="inlineStr">
         <is>
           <t>10 Decorators × 150 SKUs × 20 orders × $8 = $150K/month</t>
         </is>
@@ -4305,7 +4278,7 @@
           <t>$1,800,000</t>
         </is>
       </c>
-      <c r="C26" s="61" t="inlineStr">
+      <c r="C26" s="56" t="inlineStr">
         <is>
           <t>$150K/month × 12 months</t>
         </is>
@@ -4325,7 +4298,7 @@
           <t>$340,000</t>
         </is>
       </c>
-      <c r="C27" s="63" t="inlineStr">
+      <c r="C27" s="58" t="inlineStr">
         <is>
           <t>PoC $0 + Design Sprint $20K + MVP 1 $80K + MVP 2 $120K + MVP 3 $120K</t>
         </is>
@@ -4345,7 +4318,7 @@
           <t>~15–17 months</t>
         </is>
       </c>
-      <c r="C28" s="61" t="inlineStr">
+      <c r="C28" s="56" t="inlineStr">
         <is>
           <t>$340K investment ÷ ramping margin — reaches positive at ~Month 15–17</t>
         </is>
@@ -4541,7 +4514,7 @@
       </c>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="64" t="inlineStr">
+      <c r="A4" s="59" t="inlineStr">
         <is>
           <t>Decorators serving the USA personalized gifting market ($40–$80 AOV) cannot list genuine leather products on Printify today, forcing them to route premium transactions to PrintKK — despite its 50-unit MOQ. If we fix the taxonomy (MAT-001) and add laser engraving with 1-unit MOQ, they will consolidate their leather spend on Printify, validated at ≥$150K GMV/month within 90 days of launch.</t>
         </is>
@@ -4690,7 +4663,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="65" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SOM — Year 2</t>
         </is>
@@ -4722,7 +4695,7 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="66" t="inlineStr">
+      <c r="A12" s="61" t="inlineStr">
         <is>
           <t>SOM — Year 5</t>
         </is>
@@ -4786,17 +4759,17 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="67" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Zero structured-taxonomy player</t>
         </is>
       </c>
-      <c r="B17" s="68" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>No POD platform has leather taxonomy + FTC compliance today</t>
         </is>
       </c>
-      <c r="C17" s="40" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>12–18 month first-mover window. First to build = first to lock in Decorator catalogs</t>
         </is>
@@ -4820,17 +4793,17 @@
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="67" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Amazon demand confirmed</t>
         </is>
       </c>
-      <c r="B19" s="68" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>BULLIANT wallet: 8,365 units/mo BSR — top POD leather SKU (accio.com 2025)</t>
         </is>
       </c>
-      <c r="C19" s="40" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>The ceiling is real. New POD SKUs enter at 5–20/mo — pilot target 20/SKU is achievable</t>
         </is>
@@ -4854,17 +4827,17 @@
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="67" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>PrintKK dependency cost</t>
         </is>
       </c>
-      <c r="B21" s="68" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Decorators using PrintKK: 50-unit MOQ, no FTC compliance, no portal</t>
         </is>
       </c>
-      <c r="C21" s="40" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Every month of inaction: Decorators build their leather catalog on a competitor</t>
         </is>
@@ -4896,7 +4869,7 @@
       </c>
     </row>
     <row r="25" ht="180" customHeight="1">
-      <c r="A25" s="69" t="inlineStr">
+      <c r="A25" s="62" t="inlineStr">
         <is>
           <t>THE 5 INITIATIVES WE PROPOSE:
 ① PoC (W0 · $0) — Before writing a single line of code, the PM validates the supply side: outreach to 50 existing Printify Decorators, obtain ≥5 signed LOIs, confirm supplier SLA (1-unit MOQ, laser engraving). If no LOIs → cancel. Cost: zero.
@@ -4981,7 +4954,7 @@
           <t>≥ 5 signed Decorator LOIs + supplier confirmed</t>
         </is>
       </c>
-      <c r="G27" s="54" t="inlineStr">
+      <c r="G27" s="49" t="inlineStr">
         <is>
           <t>CANCEL — $0 spent, no engineering</t>
         </is>
@@ -5018,7 +4991,7 @@
           <t>Figma approved by FE Director + UX Lead</t>
         </is>
       </c>
-      <c r="G28" s="52" t="inlineStr">
+      <c r="G28" s="47" t="inlineStr">
         <is>
           <t>PAUSE — redesign before MVP 1 start</t>
         </is>
@@ -5062,37 +5035,37 @@
       </c>
     </row>
     <row r="30" ht="44" customHeight="1">
-      <c r="A30" s="56" t="inlineStr">
+      <c r="A30" s="51" t="inlineStr">
         <is>
           <t>MVP 2 — Mockup</t>
         </is>
       </c>
-      <c r="B30" s="57" t="inlineStr">
+      <c r="B30" s="52" t="inlineStr">
         <is>
           <t>W9–W16</t>
         </is>
       </c>
-      <c r="C30" s="57" t="inlineStr">
+      <c r="C30" s="52" t="inlineStr">
         <is>
           <t>~$120K</t>
         </is>
       </c>
-      <c r="D30" s="57" t="inlineStr">
+      <c r="D30" s="52" t="inlineStr">
         <is>
           <t>~$220K</t>
         </is>
       </c>
-      <c r="E30" s="57" t="inlineStr">
+      <c r="E30" s="52" t="inlineStr">
         <is>
           <t>Static leather texture mockup engine (3 textures/tier, assets locked W9 D1) · Decorator portal UI · AI field-assist agent · scoring UI · 5 Decorators onboarded · Shopify pilot ★</t>
         </is>
       </c>
-      <c r="F30" s="57" t="inlineStr">
+      <c r="F30" s="52" t="inlineStr">
         <is>
           <t>5 Decorators with 150 valid approved blueprints · error rate &lt; 10% · Shopify W16 signal</t>
         </is>
       </c>
-      <c r="G30" s="50" t="inlineStr">
+      <c r="G30" s="46" t="inlineStr">
         <is>
           <t>PAUSE — redesign portal UI &amp; AI flow · ⚠ 8-week critical path</t>
         </is>
@@ -5129,7 +5102,7 @@
           <t>≥ 20 orders/SKU Month 1 · Kill if &lt; 15 at Month 2</t>
         </is>
       </c>
-      <c r="G31" s="52" t="inlineStr">
+      <c r="G31" s="47" t="inlineStr">
         <is>
           <t>KILL (&lt; 15/SKU at M2) — halt &amp; reallocate team</t>
         </is>
@@ -5181,31 +5154,31 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="70" t="inlineStr">
+      <c r="A36" s="63" t="inlineStr">
         <is>
           <t>Conservative</t>
         </is>
       </c>
-      <c r="B36" s="71" t="n">
+      <c r="B36" s="64" t="n">
         <v>8</v>
       </c>
-      <c r="C36" s="72" t="n">
+      <c r="C36" s="65" t="n">
         <v>60000</v>
       </c>
-      <c r="D36" s="72" t="n">
+      <c r="D36" s="65" t="n">
         <v>720000</v>
       </c>
-      <c r="E36" s="71" t="inlineStr">
+      <c r="E36" s="64" t="inlineStr">
         <is>
           <t>&gt; 36 months</t>
         </is>
       </c>
-      <c r="F36" s="70" t="inlineStr">
+      <c r="F36" s="63" t="inlineStr">
         <is>
           <t>KILL at Month 2 Gate (&lt; 15 orders)</t>
         </is>
       </c>
-      <c r="G36" s="73" t="inlineStr">
+      <c r="G36" s="66" t="inlineStr">
         <is>
           <t>POD industry average — Printify data</t>
         </is>
@@ -5217,16 +5190,16 @@
           <t>Base Case</t>
         </is>
       </c>
-      <c r="B37" s="74" t="n">
+      <c r="B37" s="67" t="n">
         <v>20</v>
       </c>
-      <c r="C37" s="75" t="n">
+      <c r="C37" s="68" t="n">
         <v>150000</v>
       </c>
-      <c r="D37" s="75" t="n">
+      <c r="D37" s="68" t="n">
         <v>1800000</v>
       </c>
-      <c r="E37" s="74" t="inlineStr">
+      <c r="E37" s="67" t="inlineStr">
         <is>
           <t>~15–17 months</t>
         </is>
@@ -5236,38 +5209,38 @@
           <t>GO — Planning Target</t>
         </is>
       </c>
-      <c r="G37" s="47" t="inlineStr">
+      <c r="G37" s="44" t="inlineStr">
         <is>
           <t>Top-quartile Etsy leather sellers proxy</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="66" t="inlineStr">
+      <c r="A38" s="61" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="B38" s="49" t="n">
+      <c r="B38" s="45" t="n">
         <v>50</v>
       </c>
-      <c r="C38" s="76" t="n">
+      <c r="C38" s="69" t="n">
         <v>375000</v>
       </c>
-      <c r="D38" s="76" t="n">
+      <c r="D38" s="69" t="n">
         <v>4500000</v>
       </c>
-      <c r="E38" s="49" t="inlineStr">
+      <c r="E38" s="45" t="inlineStr">
         <is>
           <t>~9–10 months</t>
         </is>
       </c>
-      <c r="F38" s="66" t="inlineStr">
+      <c r="F38" s="61" t="inlineStr">
         <is>
           <t>SCALE to 1,500+ SKUs</t>
         </is>
       </c>
-      <c r="G38" s="51" t="inlineStr">
+      <c r="G38" s="40" t="inlineStr">
         <is>
           <t>Top 5% Etsy / Amazon POD performers proxy</t>
         </is>
@@ -5386,32 +5359,32 @@
           <t>Gate 0 · PoC</t>
         </is>
       </c>
-      <c r="B66" s="77" t="inlineStr">
+      <c r="B66" s="70" t="inlineStr">
         <is>
           <t>W0</t>
         </is>
       </c>
-      <c r="C66" s="77" t="inlineStr">
+      <c r="C66" s="70" t="inlineStr">
         <is>
           <t>≥ 5 Signed LOIs + Supplier SLA ready</t>
         </is>
       </c>
-      <c r="D66" s="78" t="inlineStr">
+      <c r="D66" s="71" t="inlineStr">
         <is>
           <t>Approve ~$20K for Design Sprint</t>
         </is>
       </c>
-      <c r="E66" s="79" t="inlineStr">
+      <c r="E66" s="72" t="inlineStr">
         <is>
           <t>CANCEL — $0 engineering spent</t>
         </is>
       </c>
-      <c r="F66" s="77" t="inlineStr">
+      <c r="F66" s="70" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="G66" s="77" t="inlineStr">
+      <c r="G66" s="70" t="inlineStr">
         <is>
           <t>Demand signal before any code written</t>
         </is>
@@ -5423,69 +5396,69 @@
           <t>Gate 1 · MVP 2</t>
         </is>
       </c>
-      <c r="B67" s="80" t="inlineStr">
+      <c r="B67" s="73" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="C67" s="80" t="inlineStr">
+      <c r="C67" s="73" t="inlineStr">
         <is>
           <t>150 valid SKUs; portal error &lt; 10%</t>
         </is>
       </c>
-      <c r="D67" s="81" t="inlineStr">
+      <c r="D67" s="74" t="inlineStr">
         <is>
           <t>Proceed to Marketplace Integrations</t>
         </is>
       </c>
-      <c r="E67" s="82" t="inlineStr">
+      <c r="E67" s="75" t="inlineStr">
         <is>
           <t>PAUSE — redesign portal UI &amp; AI flow</t>
         </is>
       </c>
-      <c r="F67" s="80" t="inlineStr">
+      <c r="F67" s="73" t="inlineStr">
         <is>
           <t>~$220K</t>
         </is>
       </c>
-      <c r="G67" s="80" t="inlineStr">
+      <c r="G67" s="73" t="inlineStr">
         <is>
           <t>Supply readiness before marketplace spend</t>
         </is>
       </c>
     </row>
     <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="56" t="inlineStr">
+      <c r="A68" s="51" t="inlineStr">
         <is>
           <t>Gate 2 · M2</t>
         </is>
       </c>
-      <c r="B68" s="83" t="inlineStr">
+      <c r="B68" s="76" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="C68" s="83" t="inlineStr">
+      <c r="C68" s="76" t="inlineStr">
         <is>
           <t>≥ 20 orders / SKU / month</t>
         </is>
       </c>
-      <c r="D68" s="84" t="inlineStr">
+      <c r="D68" s="77" t="inlineStr">
         <is>
           <t>FULL SCALE — expand to 1,500+ SKUs</t>
         </is>
       </c>
-      <c r="E68" s="85" t="inlineStr">
+      <c r="E68" s="78" t="inlineStr">
         <is>
           <t>KILL (&lt; 15) — halt &amp; reallocate team</t>
         </is>
       </c>
-      <c r="F68" s="83" t="inlineStr">
+      <c r="F68" s="76" t="inlineStr">
         <is>
           <t>~$340K</t>
         </is>
       </c>
-      <c r="G68" s="83" t="inlineStr">
+      <c r="G68" s="76" t="inlineStr">
         <is>
           <t>M1 has launch noise; M2 = true organic signal</t>
         </is>
@@ -5497,22 +5470,22 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="B69" s="86" t="n">
+      <c r="B69" s="79" t="n">
         <v>55</v>
       </c>
-      <c r="C69" s="87" t="n">
+      <c r="C69" s="80" t="n">
         <v>130</v>
       </c>
-      <c r="D69" s="88" t="n">
+      <c r="D69" s="81" t="n">
         <v>320</v>
       </c>
-      <c r="E69" s="89" t="n">
+      <c r="E69" s="82" t="n">
         <v>60</v>
       </c>
-      <c r="F69" s="90" t="n">
+      <c r="F69" s="81" t="n">
         <v>150</v>
       </c>
-      <c r="G69" s="91" t="n">
+      <c r="G69" s="83" t="n">
         <v>375</v>
       </c>
     </row>
@@ -5522,22 +5495,22 @@
           <t>M12</t>
         </is>
       </c>
-      <c r="B70" s="92" t="n">
+      <c r="B70" s="84" t="n">
         <v>60</v>
       </c>
-      <c r="C70" s="93" t="n">
+      <c r="C70" s="85" t="n">
         <v>150</v>
       </c>
-      <c r="D70" s="94" t="n">
+      <c r="D70" s="86" t="n">
         <v>375</v>
       </c>
-      <c r="E70" s="89" t="n">
+      <c r="E70" s="82" t="n">
         <v>60</v>
       </c>
-      <c r="F70" s="90" t="n">
+      <c r="F70" s="81" t="n">
         <v>150</v>
       </c>
-      <c r="G70" s="91" t="n">
+      <c r="G70" s="83" t="n">
         <v>375</v>
       </c>
     </row>
@@ -5586,17 +5559,17 @@
           <t>Decorators</t>
         </is>
       </c>
-      <c r="B73" s="95" t="inlineStr">
+      <c r="B73" s="87" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C73" s="96" t="inlineStr">
+      <c r="C73" s="23" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D73" s="49" t="inlineStr">
+      <c r="D73" s="45" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -5618,12 +5591,12 @@
           <t>Orders/SKU/month</t>
         </is>
       </c>
-      <c r="B74" s="97" t="inlineStr">
+      <c r="B74" s="88" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C74" s="96" t="inlineStr">
+      <c r="C74" s="23" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -5650,17 +5623,17 @@
           <t>Monthly margin</t>
         </is>
       </c>
-      <c r="B75" s="95" t="inlineStr">
+      <c r="B75" s="87" t="inlineStr">
         <is>
           <t>$60K</t>
         </is>
       </c>
-      <c r="C75" s="96" t="inlineStr">
+      <c r="C75" s="23" t="inlineStr">
         <is>
           <t>$150K</t>
         </is>
       </c>
-      <c r="D75" s="49" t="inlineStr">
+      <c r="D75" s="45" t="inlineStr">
         <is>
           <t>$375K</t>
         </is>
@@ -5682,12 +5655,12 @@
           <t>Annual run-rate</t>
         </is>
       </c>
-      <c r="B76" s="97" t="inlineStr">
+      <c r="B76" s="88" t="inlineStr">
         <is>
           <t>$720K</t>
         </is>
       </c>
-      <c r="C76" s="96" t="inlineStr">
+      <c r="C76" s="23" t="inlineStr">
         <is>
           <t>$1.8M</t>
         </is>
@@ -5714,17 +5687,17 @@
           <t>Payback period</t>
         </is>
       </c>
-      <c r="B77" s="95" t="inlineStr">
+      <c r="B77" s="87" t="inlineStr">
         <is>
           <t>&gt; 36 mo</t>
         </is>
       </c>
-      <c r="C77" s="96" t="inlineStr">
+      <c r="C77" s="23" t="inlineStr">
         <is>
           <t>~16 mo</t>
         </is>
       </c>
-      <c r="D77" s="49" t="inlineStr">
+      <c r="D77" s="45" t="inlineStr">
         <is>
           <t>~9.5 mo</t>
         </is>
@@ -5746,12 +5719,12 @@
           <t>Total investment</t>
         </is>
       </c>
-      <c r="B78" s="97" t="inlineStr">
+      <c r="B78" s="88" t="inlineStr">
         <is>
           <t>$340K</t>
         </is>
       </c>
-      <c r="C78" s="96" t="inlineStr">
+      <c r="C78" s="23" t="inlineStr">
         <is>
           <t>$340K</t>
         </is>
@@ -5773,32 +5746,32 @@
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="56" t="inlineStr">
+      <c r="A79" s="51" t="inlineStr">
         <is>
           <t>Decision at M2</t>
         </is>
       </c>
-      <c r="B79" s="71" t="inlineStr">
+      <c r="B79" s="64" t="inlineStr">
         <is>
           <t>KILL</t>
         </is>
       </c>
-      <c r="C79" s="96" t="inlineStr">
+      <c r="C79" s="23" t="inlineStr">
         <is>
           <t>GO</t>
         </is>
       </c>
-      <c r="D79" s="98" t="inlineStr">
+      <c r="D79" s="89" t="inlineStr">
         <is>
           <t>SCALE</t>
         </is>
       </c>
-      <c r="E79" s="99" t="inlineStr">
+      <c r="E79" s="90" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F79" s="99" t="inlineStr">
+      <c r="F79" s="90" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5851,7 +5824,7 @@
           <t>US leather goods market: $54.26B TAM · 6.7% CAGR</t>
         </is>
       </c>
-      <c r="C86" s="100" t="inlineStr">
+      <c r="C86" s="91" t="inlineStr">
         <is>
           <t>https://www.novaoneadvisor.com/report/us-leather-goods-market</t>
         </is>
@@ -5872,7 +5845,7 @@
           <t>Amazon USA BSR: BULLIANT leather wallet — 8,365 units/month</t>
         </is>
       </c>
-      <c r="C87" s="101" t="inlineStr">
+      <c r="C87" s="92" t="inlineStr">
         <is>
           <t>https://www.accio.com/business/amazon-mens-wallet-best-seller</t>
         </is>
@@ -5893,7 +5866,7 @@
           <t>Etsy USA: "leather" = #215 top keyword · +57% search growth Nov–Dec</t>
         </is>
       </c>
-      <c r="C88" s="100" t="inlineStr">
+      <c r="C88" s="91" t="inlineStr">
         <is>
           <t>https://erank.com</t>
         </is>
@@ -5914,7 +5887,7 @@
           <t>Etsy top-quartile leather sellers: 15–25 orders/SKU/mo · "personalized leather bag" GMV $130K–$270K/week</t>
         </is>
       </c>
-      <c r="C89" s="101" t="inlineStr">
+      <c r="C89" s="92" t="inlineStr">
         <is>
           <t>https://shelftrend.com</t>
         </is>
@@ -5935,7 +5908,7 @@
           <t>New material attribute standard enabling leather taxonomy in Shopify metafields — no indexing lag</t>
         </is>
       </c>
-      <c r="C90" s="100" t="inlineStr">
+      <c r="C90" s="91" t="inlineStr">
         <is>
           <t>https://help.shopify.com/en/manual/products/details/product-type</t>
         </is>
@@ -5956,7 +5929,7 @@
           <t>Genuine leather labeling requirements · PU/bonded cannot be labeled "genuine leather"</t>
         </is>
       </c>
-      <c r="C91" s="101" t="inlineStr">
+      <c r="C91" s="92" t="inlineStr">
         <is>
           <t>https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather</t>
         </is>
@@ -5977,7 +5950,7 @@
           <t>Competitor genuine leather POD: 50-unit MOQ · no taxonomy · no FTC compliance</t>
         </is>
       </c>
-      <c r="C92" s="100" t="inlineStr">
+      <c r="C92" s="91" t="inlineStr">
         <is>
           <t>https://printkk.com</t>
         </is>
@@ -5998,7 +5971,7 @@
           <t>All deliverables: PRD HTML, Excel workbook, demand charts, interview prep</t>
         </is>
       </c>
-      <c r="C93" s="101" t="inlineStr">
+      <c r="C93" s="92" t="inlineStr">
         <is>
           <t>https://github.com/elenacastan-maker/fyul-pm-interview-prep</t>
         </is>
@@ -6131,37 +6104,37 @@
           <t>Genuine leather products (Full-Grain / Top-Grain)</t>
         </is>
       </c>
-      <c r="B5" s="95" t="inlineStr">
+      <c r="B5" s="87" t="inlineStr">
         <is>
           <t>❌ 0</t>
         </is>
       </c>
-      <c r="C5" s="102" t="inlineStr">
+      <c r="C5" s="45" t="inlineStr">
         <is>
           <t>✅ 150+ SKUs</t>
         </is>
       </c>
-      <c r="D5" s="95" t="inlineStr">
+      <c r="D5" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E5" s="95" t="inlineStr">
+      <c r="E5" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F5" s="95" t="inlineStr">
+      <c r="F5" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G5" s="95" t="inlineStr">
+      <c r="G5" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H5" s="95" t="inlineStr">
+      <c r="H5" s="87" t="inlineStr">
         <is>
           <t>⚠ Yes, no standards</t>
         </is>
@@ -6178,7 +6151,7 @@
           <t>✅ ~45</t>
         </is>
       </c>
-      <c r="C6" s="102" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -6215,37 +6188,37 @@
           <t>Material taxonomy (tier classification)</t>
         </is>
       </c>
-      <c r="B7" s="95" t="inlineStr">
+      <c r="B7" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C7" s="102" t="inlineStr">
+      <c r="C7" s="45" t="inlineStr">
         <is>
           <t>✅ 8 fields</t>
         </is>
       </c>
-      <c r="D7" s="95" t="inlineStr">
+      <c r="D7" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E7" s="95" t="inlineStr">
+      <c r="E7" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F7" s="95" t="inlineStr">
+      <c r="F7" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G7" s="95" t="inlineStr">
+      <c r="G7" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H7" s="95" t="inlineStr">
+      <c r="H7" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6257,37 +6230,37 @@
           <t>FTC compliance / auto-reject mislabeling</t>
         </is>
       </c>
-      <c r="B8" s="97" t="inlineStr">
+      <c r="B8" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C8" s="102" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>✅ MAT-001</t>
         </is>
       </c>
-      <c r="D8" s="97" t="inlineStr">
+      <c r="D8" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E8" s="97" t="inlineStr">
+      <c r="E8" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F8" s="97" t="inlineStr">
+      <c r="F8" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G8" s="97" t="inlineStr">
+      <c r="G8" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H8" s="97" t="inlineStr">
+      <c r="H8" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6299,37 +6272,37 @@
           <t>Laser engraving support</t>
         </is>
       </c>
-      <c r="B9" s="95" t="inlineStr">
+      <c r="B9" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C9" s="102" t="inlineStr">
+      <c r="C9" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 1</t>
         </is>
       </c>
-      <c r="D9" s="95" t="inlineStr">
+      <c r="D9" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E9" s="95" t="inlineStr">
+      <c r="E9" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F9" s="95" t="inlineStr">
+      <c r="F9" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G9" s="95" t="inlineStr">
+      <c r="G9" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H9" s="49" t="inlineStr">
+      <c r="H9" s="45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -6341,37 +6314,37 @@
           <t>Debossing support</t>
         </is>
       </c>
-      <c r="B10" s="97" t="inlineStr">
+      <c r="B10" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C10" s="102" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 1</t>
         </is>
       </c>
-      <c r="D10" s="97" t="inlineStr">
+      <c r="D10" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E10" s="97" t="inlineStr">
+      <c r="E10" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F10" s="97" t="inlineStr">
+      <c r="F10" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G10" s="97" t="inlineStr">
+      <c r="G10" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H10" s="97" t="inlineStr">
+      <c r="H10" s="88" t="inlineStr">
         <is>
           <t>⚠ Partial</t>
         </is>
@@ -6383,37 +6356,37 @@
           <t>Leather mockup engine</t>
         </is>
       </c>
-      <c r="B11" s="95" t="inlineStr">
+      <c r="B11" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C11" s="102" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
       </c>
-      <c r="D11" s="49" t="inlineStr">
+      <c r="D11" s="45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E11" s="95" t="inlineStr">
+      <c r="E11" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F11" s="95" t="inlineStr">
+      <c r="F11" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G11" s="95" t="inlineStr">
+      <c r="G11" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H11" s="95" t="inlineStr">
+      <c r="H11" s="87" t="inlineStr">
         <is>
           <t>⚠ Basic</t>
         </is>
@@ -6425,37 +6398,37 @@
           <t>Decorator self-onboard portal (leather)</t>
         </is>
       </c>
-      <c r="B12" s="97" t="inlineStr">
+      <c r="B12" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C12" s="102" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
       </c>
-      <c r="D12" s="97" t="inlineStr">
+      <c r="D12" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E12" s="97" t="inlineStr">
+      <c r="E12" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F12" s="97" t="inlineStr">
+      <c r="F12" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G12" s="97" t="inlineStr">
+      <c r="G12" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H12" s="97" t="inlineStr">
+      <c r="H12" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6467,37 +6440,37 @@
           <t>AI field-assist for material attributes</t>
         </is>
       </c>
-      <c r="B13" s="95" t="inlineStr">
+      <c r="B13" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C13" s="102" t="inlineStr">
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
       </c>
-      <c r="D13" s="95" t="inlineStr">
+      <c r="D13" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E13" s="95" t="inlineStr">
+      <c r="E13" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F13" s="95" t="inlineStr">
+      <c r="F13" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G13" s="95" t="inlineStr">
+      <c r="G13" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H13" s="95" t="inlineStr">
+      <c r="H13" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6509,37 +6482,37 @@
           <t>Prop 65 auto-disclosure (CA / Amazon)</t>
         </is>
       </c>
-      <c r="B14" s="97" t="inlineStr">
+      <c r="B14" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C14" s="102" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
       </c>
-      <c r="D14" s="97" t="inlineStr">
+      <c r="D14" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E14" s="97" t="inlineStr">
+      <c r="E14" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F14" s="97" t="inlineStr">
+      <c r="F14" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G14" s="97" t="inlineStr">
+      <c r="G14" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H14" s="97" t="inlineStr">
+      <c r="H14" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6551,37 +6524,37 @@
           <t>Amazon SP-API leather category</t>
         </is>
       </c>
-      <c r="B15" s="95" t="inlineStr">
+      <c r="B15" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C15" s="102" t="inlineStr">
+      <c r="C15" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
       </c>
-      <c r="D15" s="49" t="inlineStr">
+      <c r="D15" s="45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E15" s="95" t="inlineStr">
+      <c r="E15" s="87" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="F15" s="95" t="inlineStr">
+      <c r="F15" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G15" s="95" t="inlineStr">
+      <c r="G15" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H15" s="95" t="inlineStr">
+      <c r="H15" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6593,37 +6566,37 @@
           <t>LWG / Oeko-Tex certification field</t>
         </is>
       </c>
-      <c r="B16" s="97" t="inlineStr">
+      <c r="B16" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C16" s="103" t="inlineStr">
+      <c r="C16" s="93" t="inlineStr">
         <is>
           <t>⏳ V2</t>
         </is>
       </c>
-      <c r="D16" s="97" t="inlineStr">
+      <c r="D16" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E16" s="97" t="inlineStr">
+      <c r="E16" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F16" s="97" t="inlineStr">
+      <c r="F16" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G16" s="97" t="inlineStr">
+      <c r="G16" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H16" s="97" t="inlineStr">
+      <c r="H16" s="88" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6635,37 +6608,37 @@
           <t>Etsy material attribute mapping</t>
         </is>
       </c>
-      <c r="B17" s="95" t="inlineStr">
+      <c r="B17" s="87" t="inlineStr">
         <is>
           <t>⚠ Generic</t>
         </is>
       </c>
-      <c r="C17" s="102" t="inlineStr">
+      <c r="C17" s="45" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
       </c>
-      <c r="D17" s="49" t="inlineStr">
+      <c r="D17" s="45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" s="49" t="inlineStr">
+      <c r="E17" s="45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="F17" s="95" t="inlineStr">
+      <c r="F17" s="87" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="G17" s="95" t="inlineStr">
+      <c r="G17" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H17" s="95" t="inlineStr">
+      <c r="H17" s="87" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6732,7 +6705,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="E22" s="55" t="inlineStr">
+      <c r="E22" s="50" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -6764,7 +6737,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="E23" s="53" t="inlineStr">
+      <c r="E23" s="48" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -6796,7 +6769,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="E24" s="55" t="inlineStr">
+      <c r="E24" s="50" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -6808,96 +6781,96 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="51" t="inlineStr">
         <is>
           <t>Printful</t>
         </is>
       </c>
-      <c r="B25" s="57" t="inlineStr">
+      <c r="B25" s="52" t="inlineStr">
         <is>
           <t>PU/faux</t>
         </is>
       </c>
-      <c r="C25" s="57" t="inlineStr">
+      <c r="C25" s="52" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D25" s="57" t="inlineStr">
+      <c r="D25" s="52" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E25" s="50" t="inlineStr">
+      <c r="E25" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F25" s="57" t="inlineStr">
+      <c r="F25" s="52" t="inlineStr">
         <is>
           <t>Scale advantage; could add genuine leather if they see Printify traction</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="56" t="inlineStr">
+      <c r="A26" s="51" t="inlineStr">
         <is>
           <t>PrintKK</t>
         </is>
       </c>
-      <c r="B26" s="57" t="inlineStr">
+      <c r="B26" s="52" t="inlineStr">
         <is>
           <t>Yes ✅</t>
         </is>
       </c>
-      <c r="C26" s="57" t="inlineStr">
+      <c r="C26" s="52" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D26" s="57" t="inlineStr">
+      <c r="D26" s="52" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E26" s="50" t="inlineStr">
+      <c r="E26" s="46" t="inlineStr">
         <is>
           <t>Medium–High</t>
         </is>
       </c>
-      <c r="F26" s="57" t="inlineStr">
+      <c r="F26" s="52" t="inlineStr">
         <is>
           <t>Only leather-focused POD — but zero material classification or FTC compliance. Key first-mover threat.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="67" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Printify</t>
         </is>
       </c>
-      <c r="B27" s="40" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>~45 PU ❌</t>
         </is>
       </c>
-      <c r="C27" s="40" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D27" s="40" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E27" s="40" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>N/A (us)</t>
         </is>
       </c>
-      <c r="F27" s="40" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Opportunity: first POD with structured leather taxonomy + automated FTC compliance = defensive moat</t>
         </is>
@@ -7110,37 +7083,37 @@
       <c r="G7" s="10" t="inlineStr"/>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="56" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>MVP 2 — Mockup</t>
         </is>
       </c>
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="52" t="inlineStr">
         <is>
           <t>W9–W16</t>
         </is>
       </c>
-      <c r="C8" s="57" t="inlineStr">
+      <c r="C8" s="52" t="inlineStr">
         <is>
           <t>~$120K</t>
         </is>
       </c>
-      <c r="D8" s="57" t="inlineStr">
+      <c r="D8" s="52" t="inlineStr">
         <is>
           <t>~$220K</t>
         </is>
       </c>
-      <c r="E8" s="57" t="inlineStr">
+      <c r="E8" s="52" t="inlineStr">
         <is>
           <t>Static leather texture mockup engine (3 textures/tier · assets locked W9D1) · Decorator portal (8 fields, plain-language) · AI field-assist agent · MAT-001 scoring UX · 5 Decorators complete onboarding</t>
         </is>
       </c>
-      <c r="F8" s="57" t="inlineStr">
+      <c r="F8" s="52" t="inlineStr">
         <is>
           <t>5 Decorators with 150 valid blueprints · error rate &lt; 10%</t>
         </is>
       </c>
-      <c r="G8" s="50" t="inlineStr">
+      <c r="G8" s="46" t="inlineStr">
         <is>
           <t>⚠ CRITICAL PATH — 8-week longest phase</t>
         </is>
@@ -7172,7 +7145,7 @@
           <t>Shopify metafields (W17–18) · Etsy material attr (W17–18) · Amazon LeatherType + Prop 65 SP-API (W19–22) · WooCommerce (W23–24) · 150 SKUs live · Pilot Month 1 read</t>
         </is>
       </c>
-      <c r="F9" s="52" t="inlineStr">
+      <c r="F9" s="47" t="inlineStr">
         <is>
           <t>≥ 20 orders/SKU Month 1 · KILL if &lt; 15 at Month 2</t>
         </is>
@@ -7192,196 +7165,196 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="104" t="inlineStr">
+      <c r="A13" s="94" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B13" s="105" t="inlineStr">
+      <c r="B13" s="95" t="inlineStr">
         <is>
           <t>W0</t>
         </is>
       </c>
-      <c r="C13" s="105" t="inlineStr">
+      <c r="C13" s="95" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="D13" s="105" t="inlineStr">
+      <c r="D13" s="95" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="E13" s="105" t="inlineStr">
+      <c r="E13" s="95" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F13" s="105" t="inlineStr">
+      <c r="F13" s="95" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="G13" s="105" t="inlineStr">
+      <c r="G13" s="95" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="H13" s="105" t="inlineStr">
+      <c r="H13" s="95" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="I13" s="105" t="inlineStr">
+      <c r="I13" s="95" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="J13" s="105" t="inlineStr">
+      <c r="J13" s="95" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="K13" s="105" t="inlineStr">
+      <c r="K13" s="95" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="L13" s="105" t="inlineStr">
+      <c r="L13" s="95" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="M13" s="105" t="inlineStr">
+      <c r="M13" s="95" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="N13" s="105" t="inlineStr">
+      <c r="N13" s="95" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="O13" s="105" t="inlineStr">
+      <c r="O13" s="95" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="P13" s="105" t="inlineStr">
+      <c r="P13" s="95" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="Q13" s="105" t="inlineStr">
+      <c r="Q13" s="95" t="inlineStr">
         <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="R13" s="105" t="inlineStr">
+      <c r="R13" s="95" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="S13" s="105" t="inlineStr">
+      <c r="S13" s="95" t="inlineStr">
         <is>
           <t>W17</t>
         </is>
       </c>
-      <c r="T13" s="105" t="inlineStr">
+      <c r="T13" s="95" t="inlineStr">
         <is>
           <t>W18</t>
         </is>
       </c>
-      <c r="U13" s="105" t="inlineStr">
+      <c r="U13" s="95" t="inlineStr">
         <is>
           <t>W19</t>
         </is>
       </c>
-      <c r="V13" s="105" t="inlineStr">
+      <c r="V13" s="95" t="inlineStr">
         <is>
           <t>W20</t>
         </is>
       </c>
-      <c r="W13" s="105" t="inlineStr">
+      <c r="W13" s="95" t="inlineStr">
         <is>
           <t>W21</t>
         </is>
       </c>
-      <c r="X13" s="105" t="inlineStr">
+      <c r="X13" s="95" t="inlineStr">
         <is>
           <t>W22</t>
         </is>
       </c>
-      <c r="Y13" s="105" t="inlineStr">
+      <c r="Y13" s="95" t="inlineStr">
         <is>
           <t>W23</t>
         </is>
       </c>
-      <c r="Z13" s="105" t="inlineStr">
+      <c r="Z13" s="95" t="inlineStr">
         <is>
           <t>W24</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="106" t="inlineStr">
+      <c r="A14" s="96" t="inlineStr">
         <is>
           <t>PoC</t>
         </is>
       </c>
-      <c r="B14" s="107" t="n"/>
+      <c r="B14" s="97" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="106" t="inlineStr">
+      <c r="A15" s="96" t="inlineStr">
         <is>
           <t>Design Sprint</t>
         </is>
       </c>
-      <c r="C15" s="108" t="n"/>
-      <c r="D15" s="108" t="n"/>
+      <c r="C15" s="98" t="n"/>
+      <c r="D15" s="98" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="106" t="inlineStr">
+      <c r="A16" s="96" t="inlineStr">
         <is>
           <t>MVP 1 — Schema</t>
         </is>
       </c>
-      <c r="E16" s="109" t="n"/>
-      <c r="F16" s="109" t="n"/>
-      <c r="G16" s="109" t="n"/>
-      <c r="H16" s="109" t="n"/>
-      <c r="I16" s="109" t="n"/>
-      <c r="J16" s="109" t="n"/>
+      <c r="E16" s="99" t="n"/>
+      <c r="F16" s="99" t="n"/>
+      <c r="G16" s="99" t="n"/>
+      <c r="H16" s="99" t="n"/>
+      <c r="I16" s="99" t="n"/>
+      <c r="J16" s="99" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="106" t="inlineStr">
+      <c r="A17" s="96" t="inlineStr">
         <is>
           <t>MVP 2 — Mockup</t>
         </is>
       </c>
-      <c r="K17" s="110" t="n"/>
-      <c r="L17" s="110" t="n"/>
-      <c r="M17" s="110" t="n"/>
-      <c r="N17" s="110" t="n"/>
-      <c r="O17" s="110" t="n"/>
-      <c r="P17" s="110" t="n"/>
-      <c r="Q17" s="110" t="n"/>
-      <c r="R17" s="110" t="n"/>
+      <c r="K17" s="100" t="n"/>
+      <c r="L17" s="100" t="n"/>
+      <c r="M17" s="100" t="n"/>
+      <c r="N17" s="100" t="n"/>
+      <c r="O17" s="100" t="n"/>
+      <c r="P17" s="100" t="n"/>
+      <c r="Q17" s="100" t="n"/>
+      <c r="R17" s="100" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="106" t="inlineStr">
+      <c r="A18" s="96" t="inlineStr">
         <is>
           <t>MVP 3 — Channels</t>
         </is>
       </c>
-      <c r="S18" s="111" t="n"/>
-      <c r="T18" s="111" t="n"/>
-      <c r="U18" s="111" t="n"/>
-      <c r="V18" s="111" t="n"/>
-      <c r="W18" s="111" t="n"/>
-      <c r="X18" s="111" t="n"/>
-      <c r="Y18" s="111" t="n"/>
-      <c r="Z18" s="111" t="n"/>
+      <c r="S18" s="101" t="n"/>
+      <c r="T18" s="101" t="n"/>
+      <c r="U18" s="101" t="n"/>
+      <c r="V18" s="101" t="n"/>
+      <c r="W18" s="101" t="n"/>
+      <c r="X18" s="101" t="n"/>
+      <c r="Y18" s="101" t="n"/>
+      <c r="Z18" s="101" t="n"/>
     </row>
     <row r="21" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -7557,7 +7530,7 @@
           <t>$0</t>
         </is>
       </c>
-      <c r="E50" s="55" t="inlineStr">
+      <c r="E50" s="50" t="inlineStr">
         <is>
           <t>GO / scope reduction</t>
         </is>
@@ -7589,7 +7562,7 @@
           <t>$0</t>
         </is>
       </c>
-      <c r="E51" s="53" t="inlineStr">
+      <c r="E51" s="48" t="inlineStr">
         <is>
           <t>GO to MVP 2 / fix blocker</t>
         </is>
@@ -7621,7 +7594,7 @@
           <t>$0 pre-launch</t>
         </is>
       </c>
-      <c r="E52" s="55" t="inlineStr">
+      <c r="E52" s="50" t="inlineStr">
         <is>
           <t>GO to marketplace / pivot supply model</t>
         </is>
@@ -7633,64 +7606,64 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="57" t="inlineStr">
+      <c r="A53" s="52" t="inlineStr">
         <is>
           <t>MVP 3 Month 1</t>
         </is>
       </c>
-      <c r="B53" s="57" t="inlineStr">
+      <c r="B53" s="52" t="inlineStr">
         <is>
           <t>Merchant demand at target</t>
         </is>
       </c>
-      <c r="C53" s="57" t="inlineStr">
+      <c r="C53" s="52" t="inlineStr">
         <is>
           <t>≥ 20 orders/SKU/month</t>
         </is>
       </c>
-      <c r="D53" s="57" t="inlineStr">
+      <c r="D53" s="52" t="inlineStr">
         <is>
           <t>~$24K/mo (pilot)</t>
         </is>
       </c>
-      <c r="E53" s="50" t="inlineStr">
+      <c r="E53" s="46" t="inlineStr">
         <is>
           <t>≥ 50 → scale · &lt; 15 at M2 → KILL</t>
         </is>
       </c>
-      <c r="F53" s="57" t="inlineStr">
+      <c r="F53" s="52" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="57" t="inlineStr">
+      <c r="A54" s="52" t="inlineStr">
         <is>
           <t>Month 2 Gate</t>
         </is>
       </c>
-      <c r="B54" s="57" t="inlineStr">
+      <c r="B54" s="52" t="inlineStr">
         <is>
           <t>Kill/continue/scale decision</t>
         </is>
       </c>
-      <c r="C54" s="57" t="inlineStr">
+      <c r="C54" s="52" t="inlineStr">
         <is>
           <t>≥ 20 orders/SKU (base sustained)</t>
         </is>
       </c>
-      <c r="D54" s="57" t="inlineStr">
+      <c r="D54" s="52" t="inlineStr">
         <is>
           <t>$150K+/mo (base, full scale)</t>
         </is>
       </c>
-      <c r="E54" s="50" t="inlineStr">
+      <c r="E54" s="46" t="inlineStr">
         <is>
           <t>FULL SCALE / KILL &lt; 15 → stop</t>
         </is>
       </c>
-      <c r="F54" s="57" t="inlineStr">
+      <c r="F54" s="52" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
@@ -7717,7 +7690,7 @@
           <t>$150K+/month</t>
         </is>
       </c>
-      <c r="E55" s="53" t="inlineStr">
+      <c r="E55" s="48" t="inlineStr">
         <is>
           <t>Full build GO / scope v2</t>
         </is>
@@ -7830,7 +7803,7 @@
           <t>Etsy: material attr · Amazon: LeatherType node · Shopify: metafield · FTC MAT-001 anchor</t>
         </is>
       </c>
-      <c r="F5" s="54" t="inlineStr">
+      <c r="F5" s="49" t="inlineStr">
         <is>
           <t>FTC compliance anchors on this field</t>
         </is>
@@ -7862,7 +7835,7 @@
           <t>Prop 65 trigger: chrome → auto-disclosure for CA / Amazon</t>
         </is>
       </c>
-      <c r="F6" s="52" t="inlineStr">
+      <c r="F6" s="47" t="inlineStr">
         <is>
           <t>Legal sign-off required by W10</t>
         </is>
@@ -7978,7 +7951,7 @@
           <t>Grade disambiguation: top_grain corrected vs. full_grain natural</t>
         </is>
       </c>
-      <c r="F10" s="52" t="inlineStr">
+      <c r="F10" s="47" t="inlineStr">
         <is>
           <t>Required to prevent misclassification at ingestion</t>
         </is>
@@ -8010,7 +7983,7 @@
           <t>Amazon: Prop 65 auto-disclosure · MAT-001 classifier output · listing gate</t>
         </is>
       </c>
-      <c r="F11" s="54" t="inlineStr">
+      <c r="F11" s="49" t="inlineStr">
         <is>
           <t>none = block on Amazon channel</t>
         </is>
@@ -8042,7 +8015,7 @@
           <t>ECO badge on PDP · sustainability filter · EU channel compliance</t>
         </is>
       </c>
-      <c r="F12" s="52" t="inlineStr">
+      <c r="F12" s="47" t="inlineStr">
         <is>
           <t>Requires supplier cert verification</t>
         </is>
@@ -8114,7 +8087,7 @@
           <t>Auto-approve ≥ 88% · FP rate &lt; 2%</t>
         </is>
       </c>
-      <c r="F17" s="54" t="inlineStr">
+      <c r="F17" s="49" t="inlineStr">
         <is>
           <t>FP &gt; 2%: legitimate Decorators blocked → churn · FN: PU reaches catalog → FTC risk</t>
         </is>
@@ -8146,7 +8119,7 @@
           <t>Form error rate &lt; 10% · Onboarding &lt; 24h</t>
         </is>
       </c>
-      <c r="F18" s="52" t="inlineStr">
+      <c r="F18" s="47" t="inlineStr">
         <is>
           <t>Wrong pre-fill: Decorator trusts it → incorrect material_tier → MAT-001 reject loop</t>
         </is>
@@ -8249,32 +8222,32 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="51" t="inlineStr">
         <is>
           <t>Amazon USA</t>
         </is>
       </c>
-      <c r="B25" s="57" t="inlineStr">
+      <c r="B25" s="52" t="inlineStr">
         <is>
           <t>W19–22</t>
         </is>
       </c>
-      <c r="C25" s="57" t="inlineStr">
+      <c r="C25" s="52" t="inlineStr">
         <is>
           <t>material_tier → LeatherType node · prop_65_compliant → Prop 65 auto-disclosure · chrome → mandatory disclosure</t>
         </is>
       </c>
-      <c r="D25" s="57" t="inlineStr">
+      <c r="D25" s="52" t="inlineStr">
         <is>
           <t>SP-API approval + Prop 65 legal sign-off by W10</t>
         </is>
       </c>
-      <c r="E25" s="50" t="inlineStr">
+      <c r="E25" s="46" t="inlineStr">
         <is>
           <t>⚠ SP-API approval 2–4w — apply W10</t>
         </is>
       </c>
-      <c r="F25" s="57" t="inlineStr">
+      <c r="F25" s="52" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -8309,56 +8282,56 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="112" t="inlineStr">
+      <c r="A27" s="102" t="inlineStr">
         <is>
           <t>TikTok Shop</t>
         </is>
       </c>
-      <c r="B27" s="51" t="inlineStr">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="C27" s="51" t="inlineStr">
+      <c r="C27" s="40" t="inlineStr">
         <is>
           <t>Manual disclosure (no API support for leather type yet)</t>
         </is>
       </c>
-      <c r="D27" s="51" t="inlineStr">
+      <c r="D27" s="40" t="inlineStr">
         <is>
           <t>Manual Prop 65 for CA sellers</t>
         </is>
       </c>
-      <c r="E27" s="51" t="inlineStr"/>
-      <c r="F27" s="51" t="inlineStr">
+      <c r="E27" s="40" t="inlineStr"/>
+      <c r="F27" s="40" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="113" t="inlineStr">
+      <c r="A28" s="103" t="inlineStr">
         <is>
           <t>PrestaShop</t>
         </is>
       </c>
-      <c r="B28" s="47" t="inlineStr">
+      <c r="B28" s="44" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="C28" s="47" t="inlineStr">
+      <c r="C28" s="44" t="inlineStr">
         <is>
           <t>Custom module (WC plugin base)</t>
         </is>
       </c>
-      <c r="D28" s="47" t="inlineStr">
+      <c r="D28" s="44" t="inlineStr">
         <is>
           <t>None special</t>
         </is>
       </c>
-      <c r="E28" s="47" t="inlineStr"/>
-      <c r="F28" s="47" t="inlineStr">
+      <c r="E28" s="44" t="inlineStr"/>
+      <c r="F28" s="44" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -8381,4 +8354,1019 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Sources &amp; References — Premium Leather PRD · Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="5" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Data point used in PRD</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Used in</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Nova One Advisor 2025</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>US leather goods market: $54.26B TAM · 6.7% CAGR</t>
+        </is>
+      </c>
+      <c r="C4" s="91" t="inlineStr">
+        <is>
+          <t>https://www.novaoneadvisor.com/report/us-leather-goods-market</t>
+        </is>
+      </c>
+      <c r="D4" s="93" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E4" s="40" t="inlineStr">
+        <is>
+          <t>Business Case · PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>accio.com 2025</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Amazon USA BSR: BULLIANT leather wallet — 8,365 units/month (top SKU benchmark)</t>
+        </is>
+      </c>
+      <c r="C5" s="92" t="inlineStr">
+        <is>
+          <t>https://www.accio.com/business/amazon-mens-wallet-best-seller</t>
+        </is>
+      </c>
+      <c r="D5" s="67" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" s="44" t="inlineStr">
+        <is>
+          <t>Business Case · Proxy · Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>eRank 2025</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Etsy USA: "leather" = #215 top keyword · +57% search volume growth Nov–Dec (gifting peak)</t>
+        </is>
+      </c>
+      <c r="C6" s="91" t="inlineStr">
+        <is>
+          <t>https://erank.com</t>
+        </is>
+      </c>
+      <c r="D6" s="93" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E6" s="40" t="inlineStr">
+        <is>
+          <t>Business Case · Proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>ShelfTrend 2025</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Etsy top-quartile leather sellers: 15–25 orders/SKU/mo · "personalized leather bag" GMV $130K–$270K/week</t>
+        </is>
+      </c>
+      <c r="C7" s="92" t="inlineStr">
+        <is>
+          <t>https://shelftrend.com</t>
+        </is>
+      </c>
+      <c r="D7" s="67" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E7" s="44" t="inlineStr">
+        <is>
+          <t>OKRs · Proxy · Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>FTC — Guides for Use of the Word "Leather"</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>MAT-001 labeling rules: PU/bonded leather cannot be marketed as "genuine leather" · auto-reject requirement</t>
+        </is>
+      </c>
+      <c r="C8" s="91" t="inlineStr">
+        <is>
+          <t>https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>PRD · OKRs · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Shopify Material Attributes (2025)</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>New material attribute standard enabling leather taxonomy in Shopify metafields — no indexing delay vs. Amazon</t>
+        </is>
+      </c>
+      <c r="C9" s="92" t="inlineStr">
+        <is>
+          <t>https://help.shopify.com/en/manual/products/details/product-type</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="inlineStr">
+        <is>
+          <t>Roadmap · PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Amazon SP-API — LeatherType attribute</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Amazon product type node for leather goods · Prop 65 disclosure field · SP-API approval 2–4 weeks</t>
+        </is>
+      </c>
+      <c r="C10" s="91" t="inlineStr">
+        <is>
+          <t>https://developer-docs.amazon.com/sp-api/docs/product-type-definitions-api-v2020-09-01-use-case-guide</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E10" s="40" t="inlineStr">
+        <is>
+          <t>Roadmap · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>PrintKK — public catalog</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Competitor genuine leather POD: 50-unit MOQ · no taxonomy · no FTC compliance · key first-mover gap</t>
+        </is>
+      </c>
+      <c r="C11" s="92" t="inlineStr">
+        <is>
+          <t>https://printkk.com</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E11" s="44" t="inlineStr">
+        <is>
+          <t>Competitor · Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Printify internal catalog audit</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>~45 leather products — 100% synthetic PU/faux/vegan · $0 genuine leather GMV confirmed</t>
+        </is>
+      </c>
+      <c r="C12" s="56" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E12" s="40" t="inlineStr">
+        <is>
+          <t>Business Case · OKRs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Leather Working Group (LWG)</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Environmental certification for tanneries: Gold / Silver / Bronze grades — eco_claims field V2 scope</t>
+        </is>
+      </c>
+      <c r="C13" s="92" t="inlineStr">
+        <is>
+          <t>https://www.leatherworkinggroup.com</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E13" s="44" t="inlineStr">
+        <is>
+          <t>Impl. Map · Glossary</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>GitHub — Full deliverables</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>PRD HTML, Excel model, demand charts, roadmap — public repo for Printify/FYUL review</t>
+        </is>
+      </c>
+      <c r="C14" s="91" t="inlineStr">
+        <is>
+          <t>https://github.com/elenacastan-maker/fyul-pm-interview-prep</t>
+        </is>
+      </c>
+      <c r="D14" s="93" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E14" s="40" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Glossary — Key Terms · Premium Leather PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="5" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Full name / context</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Where used</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>POD</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="inlineStr">
+        <is>
+          <t>Print on Demand</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Manufacturing model where products are made only after an order is placed — no inventory held by the seller. Printify operates as a POD marketplace.</t>
+        </is>
+      </c>
+      <c r="D4" s="104" t="inlineStr">
+        <is>
+          <t>Throughout</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Decorator</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>Printify seller</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Printify's term for a merchant who designs products on the platform, sets prices, and sells through their own storefront. Decorators do not hold inventory.</t>
+        </is>
+      </c>
+      <c r="D5" s="105" t="inlineStr">
+        <is>
+          <t>Throughout</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Blueprint</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Printify product template</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>A Printify template that defines the base product, customization area, print provider, and pricing. Decorators create listings from blueprints.</t>
+        </is>
+      </c>
+      <c r="D6" s="104" t="inlineStr">
+        <is>
+          <t>PRD · OKRs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>Stock Keeping Unit</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>A unique identifier for a specific product variant (e.g. a black full-grain leather wallet, laser-engraved). Used to track sales velocity per listing.</t>
+        </is>
+      </c>
+      <c r="D7" s="105" t="inlineStr">
+        <is>
+          <t>Throughout</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Gross Merchandise Value</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Total value of orders processed through the platform before fees, refunds, or chargebacks. Platform margin = GMV × take rate.</t>
+        </is>
+      </c>
+      <c r="D8" s="104" t="inlineStr">
+        <is>
+          <t>Business Case · OKRs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>AOV</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Average revenue per completed transaction. Premium leather AOV: $45–65 vs. $18–25 for apparel — key driver of the $8/order margin assumption.</t>
+        </is>
+      </c>
+      <c r="D9" s="105" t="inlineStr">
+        <is>
+          <t>Business Case · Proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>MOQ</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Minimum Order Quantity</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Minimum number of units a supplier requires per order. PrintKK requires 50-unit MOQ; Printify's 1-unit MOQ is a key competitive differentiator.</t>
+        </is>
+      </c>
+      <c r="D10" s="104" t="inlineStr">
+        <is>
+          <t>Competitor · Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>TAM</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>Total Addressable Market</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>The total global demand for a product category if there were no competition or constraints. US leather goods TAM: $54.26B (Nova One Advisor 2025).</t>
+        </is>
+      </c>
+      <c r="D11" s="105" t="inlineStr">
+        <is>
+          <t>Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>Serviceable Addressable Market</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>The portion of TAM that a business can realistically target given its model. For Printify: personalized/custom leather goods sold online via POD.</t>
+        </is>
+      </c>
+      <c r="D12" s="104" t="inlineStr">
+        <is>
+          <t>Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>SOM</t>
+        </is>
+      </c>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>Serviceable Obtainable Market</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>The portion of SAM a company can realistically capture. Modeled as Printify's leather category revenue at pilot scale → full scale.</t>
+        </is>
+      </c>
+      <c r="D13" s="105" t="inlineStr">
+        <is>
+          <t>Business Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>BSR</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t>Best Seller Rank (Amazon)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Amazon's ranking of products by sales velocity within a category. Used as a demand proxy: BULLIANT leather wallet BSR = 8,365 units/month.</t>
+        </is>
+      </c>
+      <c r="D14" s="104" t="inlineStr">
+        <is>
+          <t>Proxy Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>FTC</t>
+        </is>
+      </c>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t>Federal Trade Commission (US)</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>US regulatory body enforcing truthful product labeling. The FTC Guides for Textile &amp; Leather (MAT-001) require accurate leather grade disclosure.</t>
+        </is>
+      </c>
+      <c r="D15" s="105" t="inlineStr">
+        <is>
+          <t>PRD · OKRs · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>FTC Leather Labeling Standard</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>The FTC guide prohibiting bonded, split, or PU leather from being labeled "genuine leather." Violation risk: product delisting + fines. The AI classifier enforces this at ingestion.</t>
+        </is>
+      </c>
+      <c r="D16" s="104" t="inlineStr">
+        <is>
+          <t>PRD · OKRs · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>Prop 65</t>
+        </is>
+      </c>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>California Proposition 65</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>California law requiring businesses to warn consumers about significant exposures to chemicals causing cancer or reproductive harm. Chrome-tanned leather may trigger Prop 65 disclosure on Amazon.</t>
+        </is>
+      </c>
+      <c r="D17" s="105" t="inlineStr">
+        <is>
+          <t>Impl. Map · Roadmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>LWG</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="inlineStr">
+        <is>
+          <t>Leather Working Group</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>International certification body for environmentally responsible leather production. Grades: Gold / Silver / Bronze. Referenced in eco_claims schema field (V2 scope).</t>
+        </is>
+      </c>
+      <c r="D18" s="104" t="inlineStr">
+        <is>
+          <t>Impl. Map · References</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>Oeko-Tex</t>
+        </is>
+      </c>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>Oeko-Tex Standard 100</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>International certification confirming leather/textiles are free from harmful substances. Relevant for eco_claims field and EU market compliance.</t>
+        </is>
+      </c>
+      <c r="D19" s="105" t="inlineStr">
+        <is>
+          <t>Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>REACH</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>EU Chemical Regulation</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>EU regulation restricting hazardous substances in products. Relevant for chrome-tanned leather sold in EU — Cr(VI) limits apply.</t>
+        </is>
+      </c>
+      <c r="D20" s="104" t="inlineStr">
+        <is>
+          <t>Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>SP-API</t>
+        </is>
+      </c>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t>Amazon Selling Partner API</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Amazon's API for marketplace integrations. Printify must apply for SP-API approval (~2–4 weeks) to list leather products with LeatherType node and Prop 65 auto-disclosure.</t>
+        </is>
+      </c>
+      <c r="D21" s="105" t="inlineStr">
+        <is>
+          <t>Roadmap · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Shopify metafield</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="inlineStr">
+        <is>
+          <t>Shopify custom product field</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Custom data fields extending Shopify product records beyond standard attributes. Printify uses these to pass material attributes (leather_grade, tanning_method) to Shopify channel. No indexing lag vs. Amazon.</t>
+        </is>
+      </c>
+      <c r="D22" s="104" t="inlineStr">
+        <is>
+          <t>Roadmap · PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>leather_grade</t>
+        </is>
+      </c>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>Schema field — quality tier</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Core material classification: full_grain / top_grain / corrected_grain / split / bonded / pu / vegan. Anchors FTC MAT-001 compliance and marketplace category routing.</t>
+        </is>
+      </c>
+      <c r="D23" s="105" t="inlineStr">
+        <is>
+          <t>PRD · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>tanning_method</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>Schema field — production method</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>How the hide was treated: vegetable / chrome / chrome_free / combination. Chrome triggers Prop 65 auto-disclosure on Amazon.</t>
+        </is>
+      </c>
+      <c r="D24" s="104" t="inlineStr">
+        <is>
+          <t>PRD · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>grain_correction</t>
+        </is>
+      </c>
+      <c r="B25" s="44" t="inlineStr">
+        <is>
+          <t>Schema field — surface treatment</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Boolean: true = corrected (sanded) grain surface, false = natural grain. Required to prevent misclassifying corrected top_grain as full_grain.</t>
+        </is>
+      </c>
+      <c r="D25" s="105" t="inlineStr">
+        <is>
+          <t>PRD · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>compliance_cert</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t>Schema field — compliance status</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Array enum: ftc_genuine / prop_65_ca / mat_001_approved / none. Drives listing gate logic — "none" blocks listing on Amazon channel.</t>
+        </is>
+      </c>
+      <c r="D26" s="104" t="inlineStr">
+        <is>
+          <t>PRD · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="33" t="inlineStr">
+        <is>
+          <t>eco_claims</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="inlineStr">
+        <is>
+          <t>Schema field — sustainability</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Array enum: lwg_gold / lwg_silver / oeko_tex / reach_compliant / none. MVP 2 scope — powers ECO badge on PDP and EU channel compliance.</t>
+        </is>
+      </c>
+      <c r="D27" s="105" t="inlineStr">
+        <is>
+          <t>PRD · Impl. Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Kill gate</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="inlineStr">
+        <is>
+          <t>Investment decision trigger</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>A predefined performance threshold that, if not met, triggers immediate halt of investment. This PRD's kill gate: &lt;15 orders/SKU at Month 2 post-launch → halt &amp; reallocate team.</t>
+        </is>
+      </c>
+      <c r="D28" s="104" t="inlineStr">
+        <is>
+          <t>Throughout</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="33" t="inlineStr">
+        <is>
+          <t>Phase gate</t>
+        </is>
+      </c>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Stage-gate decision framework</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>A structured decision point between project phases where continuation is contingent on meeting predefined criteria. Each phase must earn the right to spend the next budget tranche.</t>
+        </is>
+      </c>
+      <c r="D29" s="105" t="inlineStr">
+        <is>
+          <t>Throughout</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Field-assist agent</t>
+        </is>
+      </c>
+      <c r="B30" s="40" t="inlineStr">
+        <is>
+          <t>AI pre-fill tool</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>A native AI agent that reads a supplier's product name + data sheet and pre-fills the 8 schema fields. Reduces form error rate from ~20–35% (unassisted) to &lt;10%.</t>
+        </is>
+      </c>
+      <c r="D30" s="104" t="inlineStr">
+        <is>
+          <t>PRD · OKRs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: fix links using =HYPERLINK() formula — works in Excel and Google Sheets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/FYUL_Leather_Financial_Model.xlsx
+++ b/deliverables/FYUL_Leather_Financial_Model.xlsx
@@ -270,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -410,10 +410,10 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -516,12 +516,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3775,10 +3769,9 @@
           <t>#215 top search term · $35–$70 AOV · 125%+ CTR</t>
         </is>
       </c>
-      <c r="D5" s="48" t="inlineStr">
-        <is>
-          <t>ShelfTrend 2025</t>
-        </is>
+      <c r="D5" s="48">
+        <f>HYPERLINK("https://shelftrend.com","ShelfTrend 2025")</f>
+        <v/>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
@@ -3807,10 +3800,9 @@
           <t>$130K–$270K / week</t>
         </is>
       </c>
-      <c r="D6" s="49" t="inlineStr">
-        <is>
-          <t>ShelfTrend 2025</t>
-        </is>
+      <c r="D6" s="49">
+        <f>HYPERLINK("https://shelftrend.com","ShelfTrend 2025")</f>
+        <v/>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -3839,10 +3831,9 @@
           <t>BULLIANT wallet — 8,365 units / month (BSR rank)</t>
         </is>
       </c>
-      <c r="D7" s="48" t="inlineStr">
-        <is>
-          <t>accio.com 2025</t>
-        </is>
+      <c r="D7" s="48">
+        <f>HYPERLINK("https://www.accio.com/business/amazon-mens-wallet-best-seller","accio.com 2025")</f>
+        <v/>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
@@ -3871,10 +3862,9 @@
           <t>$54.26B total · 6.7% CAGR · custom/POD ~$2B addressable (est.)</t>
         </is>
       </c>
-      <c r="D8" s="49" t="inlineStr">
-        <is>
-          <t>Nova One Advisor 2025</t>
-        </is>
+      <c r="D8" s="49">
+        <f>HYPERLINK("https://www.novaoneadvisor.com/report/us-leather-goods-market","Nova One Advisor 2025")</f>
+        <v/>
       </c>
       <c r="E8" s="41" t="inlineStr">
         <is>
@@ -3967,10 +3957,9 @@
           <t>#215 top keyword · +57% search volume growth Nov–Dec (gifting peak)</t>
         </is>
       </c>
-      <c r="D11" s="48" t="inlineStr">
-        <is>
-          <t>eRank 2025</t>
-        </is>
+      <c r="D11" s="48">
+        <f>HYPERLINK("https://erank.com","eRank 2025")</f>
+        <v/>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
@@ -3999,10 +3988,9 @@
           <t>50-unit minimum order · no taxonomy fields · no FTC compliance</t>
         </is>
       </c>
-      <c r="D12" s="49" t="inlineStr">
-        <is>
-          <t>Public pricing (printKK.com)</t>
-        </is>
+      <c r="D12" s="49">
+        <f>HYPERLINK("https://printkk.com","Public pricing (printKK.com)")</f>
+        <v/>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
@@ -4422,16 +4410,8 @@
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="C28:F28"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5792,10 +5772,9 @@
           <t>US leather goods market: $54.26B TAM · 6.7% CAGR</t>
         </is>
       </c>
-      <c r="C86" s="84" t="inlineStr">
-        <is>
-          <t>https://www.novaoneadvisor.com/report/us-leather-goods-market</t>
-        </is>
+      <c r="C86" s="48">
+        <f>HYPERLINK("https://www.novaoneadvisor.com/report/us-leather-goods-market","https://www.novaoneadvisor.com/report/us-leather-goods-market")</f>
+        <v/>
       </c>
       <c r="D86" s="31" t="n"/>
       <c r="E86" s="31" t="n"/>
@@ -5813,10 +5792,9 @@
           <t>Amazon USA BSR: BULLIANT leather wallet — 8,365 units/month</t>
         </is>
       </c>
-      <c r="C87" s="85" t="inlineStr">
-        <is>
-          <t>https://www.accio.com/business/amazon-mens-wallet-best-seller</t>
-        </is>
+      <c r="C87" s="49">
+        <f>HYPERLINK("https://www.accio.com/business/amazon-mens-wallet-best-seller","https://www.accio.com/business/amazon-mens-wallet-best-seller")</f>
+        <v/>
       </c>
       <c r="D87" s="31" t="n"/>
       <c r="E87" s="31" t="n"/>
@@ -5834,10 +5812,9 @@
           <t>Etsy USA: "leather" = #215 top keyword · +57% search growth Nov–Dec</t>
         </is>
       </c>
-      <c r="C88" s="84" t="inlineStr">
-        <is>
-          <t>https://erank.com</t>
-        </is>
+      <c r="C88" s="48">
+        <f>HYPERLINK("https://erank.com","https://erank.com")</f>
+        <v/>
       </c>
       <c r="D88" s="31" t="n"/>
       <c r="E88" s="31" t="n"/>
@@ -5855,10 +5832,9 @@
           <t>Etsy top-quartile leather sellers: 15–25 orders/SKU/mo · "personalized leather bag" GMV $130K–$270K/week</t>
         </is>
       </c>
-      <c r="C89" s="85" t="inlineStr">
-        <is>
-          <t>https://shelftrend.com</t>
-        </is>
+      <c r="C89" s="49">
+        <f>HYPERLINK("https://shelftrend.com","https://shelftrend.com")</f>
+        <v/>
       </c>
       <c r="D89" s="31" t="n"/>
       <c r="E89" s="31" t="n"/>
@@ -5876,10 +5852,9 @@
           <t>New material attribute standard enabling leather taxonomy in Shopify metafields — no indexing lag</t>
         </is>
       </c>
-      <c r="C90" s="84" t="inlineStr">
-        <is>
-          <t>https://help.shopify.com/en/manual/products/details/product-type</t>
-        </is>
+      <c r="C90" s="48">
+        <f>HYPERLINK("https://help.shopify.com/en/manual/products/details/product-type","https://help.shopify.com/en/manual/products/details/product-type")</f>
+        <v/>
       </c>
       <c r="D90" s="31" t="n"/>
       <c r="E90" s="31" t="n"/>
@@ -5897,10 +5872,9 @@
           <t>Genuine leather labeling requirements · PU/bonded cannot be labeled "genuine leather"</t>
         </is>
       </c>
-      <c r="C91" s="85" t="inlineStr">
-        <is>
-          <t>https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather</t>
-        </is>
+      <c r="C91" s="49">
+        <f>HYPERLINK("https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather","https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather")</f>
+        <v/>
       </c>
       <c r="D91" s="31" t="n"/>
       <c r="E91" s="31" t="n"/>
@@ -5918,10 +5892,9 @@
           <t>Competitor genuine leather POD: 50-unit MOQ · no taxonomy · no FTC compliance</t>
         </is>
       </c>
-      <c r="C92" s="84" t="inlineStr">
-        <is>
-          <t>https://printkk.com</t>
-        </is>
+      <c r="C92" s="48">
+        <f>HYPERLINK("https://printkk.com","https://printkk.com")</f>
+        <v/>
       </c>
       <c r="D92" s="31" t="n"/>
       <c r="E92" s="31" t="n"/>
@@ -5939,10 +5912,9 @@
           <t>All deliverables: PRD HTML, Excel workbook, demand charts, interview prep</t>
         </is>
       </c>
-      <c r="C93" s="85" t="inlineStr">
-        <is>
-          <t>https://github.com/elenacastan-maker/fyul-pm-interview-prep</t>
-        </is>
+      <c r="C93" s="49">
+        <f>HYPERLINK("https://github.com/elenacastan-maker/fyul-pm-interview-prep","https://github.com/elenacastan-maker/fyul-pm-interview-prep")</f>
+        <v/>
       </c>
       <c r="D93" s="31" t="n"/>
       <c r="E93" s="31" t="n"/>
@@ -5975,18 +5947,8 @@
     <mergeCell ref="A71:G71"/>
     <mergeCell ref="C87:G87"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId8"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6539,7 +6501,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C16" s="86" t="inlineStr">
+      <c r="C16" s="84" t="inlineStr">
         <is>
           <t>⏳ V2</t>
         </is>
@@ -7133,196 +7095,196 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="87" t="inlineStr">
+      <c r="A13" s="85" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B13" s="88" t="inlineStr">
+      <c r="B13" s="86" t="inlineStr">
         <is>
           <t>W0</t>
         </is>
       </c>
-      <c r="C13" s="88" t="inlineStr">
+      <c r="C13" s="86" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="D13" s="88" t="inlineStr">
+      <c r="D13" s="86" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="E13" s="88" t="inlineStr">
+      <c r="E13" s="86" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F13" s="88" t="inlineStr">
+      <c r="F13" s="86" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="G13" s="88" t="inlineStr">
+      <c r="G13" s="86" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="H13" s="88" t="inlineStr">
+      <c r="H13" s="86" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="I13" s="88" t="inlineStr">
+      <c r="I13" s="86" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="J13" s="88" t="inlineStr">
+      <c r="J13" s="86" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="K13" s="88" t="inlineStr">
+      <c r="K13" s="86" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="L13" s="88" t="inlineStr">
+      <c r="L13" s="86" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="M13" s="88" t="inlineStr">
+      <c r="M13" s="86" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="N13" s="88" t="inlineStr">
+      <c r="N13" s="86" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="O13" s="88" t="inlineStr">
+      <c r="O13" s="86" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="P13" s="88" t="inlineStr">
+      <c r="P13" s="86" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="Q13" s="88" t="inlineStr">
+      <c r="Q13" s="86" t="inlineStr">
         <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="R13" s="88" t="inlineStr">
+      <c r="R13" s="86" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="S13" s="88" t="inlineStr">
+      <c r="S13" s="86" t="inlineStr">
         <is>
           <t>W17</t>
         </is>
       </c>
-      <c r="T13" s="88" t="inlineStr">
+      <c r="T13" s="86" t="inlineStr">
         <is>
           <t>W18</t>
         </is>
       </c>
-      <c r="U13" s="88" t="inlineStr">
+      <c r="U13" s="86" t="inlineStr">
         <is>
           <t>W19</t>
         </is>
       </c>
-      <c r="V13" s="88" t="inlineStr">
+      <c r="V13" s="86" t="inlineStr">
         <is>
           <t>W20</t>
         </is>
       </c>
-      <c r="W13" s="88" t="inlineStr">
+      <c r="W13" s="86" t="inlineStr">
         <is>
           <t>W21</t>
         </is>
       </c>
-      <c r="X13" s="88" t="inlineStr">
+      <c r="X13" s="86" t="inlineStr">
         <is>
           <t>W22</t>
         </is>
       </c>
-      <c r="Y13" s="88" t="inlineStr">
+      <c r="Y13" s="86" t="inlineStr">
         <is>
           <t>W23</t>
         </is>
       </c>
-      <c r="Z13" s="88" t="inlineStr">
+      <c r="Z13" s="86" t="inlineStr">
         <is>
           <t>W24</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="89" t="inlineStr">
+      <c r="A14" s="87" t="inlineStr">
         <is>
           <t>PoC</t>
         </is>
       </c>
-      <c r="B14" s="90" t="n"/>
+      <c r="B14" s="88" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="89" t="inlineStr">
+      <c r="A15" s="87" t="inlineStr">
         <is>
           <t>Design Sprint</t>
         </is>
       </c>
-      <c r="C15" s="91" t="n"/>
-      <c r="D15" s="91" t="n"/>
+      <c r="C15" s="89" t="n"/>
+      <c r="D15" s="89" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="89" t="inlineStr">
+      <c r="A16" s="87" t="inlineStr">
         <is>
           <t>MVP 1 — Schema</t>
         </is>
       </c>
-      <c r="E16" s="92" t="n"/>
-      <c r="F16" s="92" t="n"/>
-      <c r="G16" s="92" t="n"/>
-      <c r="H16" s="92" t="n"/>
-      <c r="I16" s="92" t="n"/>
-      <c r="J16" s="92" t="n"/>
+      <c r="E16" s="90" t="n"/>
+      <c r="F16" s="90" t="n"/>
+      <c r="G16" s="90" t="n"/>
+      <c r="H16" s="90" t="n"/>
+      <c r="I16" s="90" t="n"/>
+      <c r="J16" s="90" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="89" t="inlineStr">
+      <c r="A17" s="87" t="inlineStr">
         <is>
           <t>MVP 2 — Mockup</t>
         </is>
       </c>
-      <c r="K17" s="93" t="n"/>
-      <c r="L17" s="93" t="n"/>
-      <c r="M17" s="93" t="n"/>
-      <c r="N17" s="93" t="n"/>
-      <c r="O17" s="93" t="n"/>
-      <c r="P17" s="93" t="n"/>
-      <c r="Q17" s="93" t="n"/>
-      <c r="R17" s="93" t="n"/>
+      <c r="K17" s="91" t="n"/>
+      <c r="L17" s="91" t="n"/>
+      <c r="M17" s="91" t="n"/>
+      <c r="N17" s="91" t="n"/>
+      <c r="O17" s="91" t="n"/>
+      <c r="P17" s="91" t="n"/>
+      <c r="Q17" s="91" t="n"/>
+      <c r="R17" s="91" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="89" t="inlineStr">
+      <c r="A18" s="87" t="inlineStr">
         <is>
           <t>MVP 3 — Channels</t>
         </is>
       </c>
-      <c r="S18" s="94" t="n"/>
-      <c r="T18" s="94" t="n"/>
-      <c r="U18" s="94" t="n"/>
-      <c r="V18" s="94" t="n"/>
-      <c r="W18" s="94" t="n"/>
-      <c r="X18" s="94" t="n"/>
-      <c r="Y18" s="94" t="n"/>
-      <c r="Z18" s="94" t="n"/>
+      <c r="S18" s="92" t="n"/>
+      <c r="T18" s="92" t="n"/>
+      <c r="U18" s="92" t="n"/>
+      <c r="V18" s="92" t="n"/>
+      <c r="W18" s="92" t="n"/>
+      <c r="X18" s="92" t="n"/>
+      <c r="Y18" s="92" t="n"/>
+      <c r="Z18" s="92" t="n"/>
     </row>
     <row r="21" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -8250,7 +8212,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="95" t="inlineStr">
+      <c r="A27" s="93" t="inlineStr">
         <is>
           <t>TikTok Shop</t>
         </is>
@@ -8278,7 +8240,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="96" t="inlineStr">
+      <c r="A28" s="94" t="inlineStr">
         <is>
           <t>PrestaShop</t>
         </is>
@@ -8386,12 +8348,11 @@
           <t>US leather goods market: $54.26B TAM · 6.7% CAGR</t>
         </is>
       </c>
-      <c r="C4" s="84" t="inlineStr">
-        <is>
-          <t>https://www.novaoneadvisor.com/report/us-leather-goods-market</t>
-        </is>
-      </c>
-      <c r="D4" s="86" t="inlineStr">
+      <c r="C4" s="48">
+        <f>HYPERLINK("https://www.novaoneadvisor.com/report/us-leather-goods-market","https://www.novaoneadvisor.com/report/us-leather-goods-market")</f>
+        <v/>
+      </c>
+      <c r="D4" s="84" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -8413,10 +8374,9 @@
           <t>Amazon USA BSR: BULLIANT leather wallet — 8,365 units/month (top SKU benchmark)</t>
         </is>
       </c>
-      <c r="C5" s="85" t="inlineStr">
-        <is>
-          <t>https://www.accio.com/business/amazon-mens-wallet-best-seller</t>
-        </is>
+      <c r="C5" s="49">
+        <f>HYPERLINK("https://www.accio.com/business/amazon-mens-wallet-best-seller","https://www.accio.com/business/amazon-mens-wallet-best-seller")</f>
+        <v/>
       </c>
       <c r="D5" s="60" t="inlineStr">
         <is>
@@ -8440,12 +8400,11 @@
           <t>Etsy USA: "leather" = #215 top keyword · +57% search volume growth Nov–Dec (gifting peak)</t>
         </is>
       </c>
-      <c r="C6" s="84" t="inlineStr">
-        <is>
-          <t>https://erank.com</t>
-        </is>
-      </c>
-      <c r="D6" s="86" t="inlineStr">
+      <c r="C6" s="48">
+        <f>HYPERLINK("https://erank.com","https://erank.com")</f>
+        <v/>
+      </c>
+      <c r="D6" s="84" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -8467,10 +8426,9 @@
           <t>Etsy top-quartile leather sellers: 15–25 orders/SKU/mo · "personalized leather bag" GMV $130K–$270K/week</t>
         </is>
       </c>
-      <c r="C7" s="85" t="inlineStr">
-        <is>
-          <t>https://shelftrend.com</t>
-        </is>
+      <c r="C7" s="49">
+        <f>HYPERLINK("https://shelftrend.com","https://shelftrend.com")</f>
+        <v/>
       </c>
       <c r="D7" s="60" t="inlineStr">
         <is>
@@ -8494,10 +8452,9 @@
           <t>MAT-001 labeling rules: PU/bonded leather cannot be marketed as "genuine leather" · auto-reject requirement</t>
         </is>
       </c>
-      <c r="C8" s="84" t="inlineStr">
-        <is>
-          <t>https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather</t>
-        </is>
+      <c r="C8" s="48">
+        <f>HYPERLINK("https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather","https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather")</f>
+        <v/>
       </c>
       <c r="D8" s="39" t="inlineStr">
         <is>
@@ -8521,10 +8478,9 @@
           <t>New material attribute standard enabling leather taxonomy in Shopify metafields — no indexing delay vs. Amazon</t>
         </is>
       </c>
-      <c r="C9" s="85" t="inlineStr">
-        <is>
-          <t>https://help.shopify.com/en/manual/products/details/product-type</t>
-        </is>
+      <c r="C9" s="49">
+        <f>HYPERLINK("https://help.shopify.com/en/manual/products/details/product-type","https://help.shopify.com/en/manual/products/details/product-type")</f>
+        <v/>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
@@ -8548,10 +8504,9 @@
           <t>Amazon product type node for leather goods · Prop 65 disclosure field · SP-API approval 2–4 weeks</t>
         </is>
       </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>https://developer-docs.amazon.com/sp-api/docs/product-type-definitions-api-v2020-09-01-use-case-guide</t>
-        </is>
+      <c r="C10" s="48">
+        <f>HYPERLINK("https://developer-docs.amazon.com/sp-api/docs/product-type-definitions-api-v2020-09-01-use-case-guide","https://developer-docs.amazon.com/sp-api/docs/product-type-definitions-api-v2020-09-01-use-case-guide")</f>
+        <v/>
       </c>
       <c r="D10" s="39" t="inlineStr">
         <is>
@@ -8575,10 +8530,9 @@
           <t>Competitor genuine leather POD: 50-unit MOQ · no taxonomy · no FTC compliance · key first-mover gap</t>
         </is>
       </c>
-      <c r="C11" s="85" t="inlineStr">
-        <is>
-          <t>https://printkk.com</t>
-        </is>
+      <c r="C11" s="49">
+        <f>HYPERLINK("https://printkk.com","https://printkk.com")</f>
+        <v/>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
@@ -8629,10 +8583,9 @@
           <t>Environmental certification for tanneries: Gold / Silver / Bronze grades — eco_claims field V2 scope</t>
         </is>
       </c>
-      <c r="C13" s="85" t="inlineStr">
-        <is>
-          <t>https://www.leatherworkinggroup.com</t>
-        </is>
+      <c r="C13" s="49">
+        <f>HYPERLINK("https://www.leatherworkinggroup.com","https://www.leatherworkinggroup.com")</f>
+        <v/>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
@@ -8656,12 +8609,11 @@
           <t>PRD HTML, Excel model, demand charts, roadmap — public repo for Printify/FYUL review</t>
         </is>
       </c>
-      <c r="C14" s="84" t="inlineStr">
-        <is>
-          <t>https://github.com/elenacastan-maker/fyul-pm-interview-prep</t>
-        </is>
-      </c>
-      <c r="D14" s="86" t="inlineStr">
+      <c r="C14" s="48">
+        <f>HYPERLINK("https://github.com/elenacastan-maker/fyul-pm-interview-prep","https://github.com/elenacastan-maker/fyul-pm-interview-prep")</f>
+        <v/>
+      </c>
+      <c r="D14" s="84" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -8676,18 +8628,6 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8753,7 +8693,7 @@
           <t>Manufacturing model where products are made only after an order is placed — no inventory held by the seller. Printify operates as a POD marketplace.</t>
         </is>
       </c>
-      <c r="D4" s="97" t="inlineStr">
+      <c r="D4" s="95" t="inlineStr">
         <is>
           <t>Throughout</t>
         </is>
@@ -8775,7 +8715,7 @@
           <t>Printify's term for a merchant who designs products on the platform, sets prices, and sells through their own storefront. Decorators do not hold inventory.</t>
         </is>
       </c>
-      <c r="D5" s="98" t="inlineStr">
+      <c r="D5" s="96" t="inlineStr">
         <is>
           <t>Throughout</t>
         </is>
@@ -8797,7 +8737,7 @@
           <t>A Printify template that defines the base product, customization area, print provider, and pricing. Decorators create listings from blueprints.</t>
         </is>
       </c>
-      <c r="D6" s="97" t="inlineStr">
+      <c r="D6" s="95" t="inlineStr">
         <is>
           <t>PRD · OKRs</t>
         </is>
@@ -8819,7 +8759,7 @@
           <t>A unique identifier for a specific product variant (e.g. a black full-grain leather wallet, laser-engraved). Used to track sales velocity per listing.</t>
         </is>
       </c>
-      <c r="D7" s="98" t="inlineStr">
+      <c r="D7" s="96" t="inlineStr">
         <is>
           <t>Throughout</t>
         </is>
@@ -8841,7 +8781,7 @@
           <t>Total value of orders processed through the platform before fees, refunds, or chargebacks. Platform margin = GMV × take rate.</t>
         </is>
       </c>
-      <c r="D8" s="97" t="inlineStr">
+      <c r="D8" s="95" t="inlineStr">
         <is>
           <t>Business Case · OKRs</t>
         </is>
@@ -8863,7 +8803,7 @@
           <t>Average revenue per completed transaction. Premium leather AOV: $45–65 vs. $18–25 for apparel — key driver of the $8/order margin assumption.</t>
         </is>
       </c>
-      <c r="D9" s="98" t="inlineStr">
+      <c r="D9" s="96" t="inlineStr">
         <is>
           <t>Business Case · Proxy</t>
         </is>
@@ -8885,7 +8825,7 @@
           <t>Minimum number of units a supplier requires per order. PrintKK requires 50-unit MOQ; Printify's 1-unit MOQ is a key competitive differentiator.</t>
         </is>
       </c>
-      <c r="D10" s="97" t="inlineStr">
+      <c r="D10" s="95" t="inlineStr">
         <is>
           <t>Competitor · Business Case</t>
         </is>
@@ -8907,7 +8847,7 @@
           <t>The total global demand for a product category if there were no competition or constraints. US leather goods TAM: $54.26B (Nova One Advisor 2025).</t>
         </is>
       </c>
-      <c r="D11" s="98" t="inlineStr">
+      <c r="D11" s="96" t="inlineStr">
         <is>
           <t>Business Case</t>
         </is>
@@ -8929,7 +8869,7 @@
           <t>The portion of TAM that a business can realistically target given its model. For Printify: personalized/custom leather goods sold online via POD.</t>
         </is>
       </c>
-      <c r="D12" s="97" t="inlineStr">
+      <c r="D12" s="95" t="inlineStr">
         <is>
           <t>Business Case</t>
         </is>
@@ -8951,7 +8891,7 @@
           <t>The portion of SAM a company can realistically capture. Modeled as Printify's leather category revenue at pilot scale → full scale.</t>
         </is>
       </c>
-      <c r="D13" s="98" t="inlineStr">
+      <c r="D13" s="96" t="inlineStr">
         <is>
           <t>Business Case</t>
         </is>
@@ -8973,7 +8913,7 @@
           <t>Amazon's ranking of products by sales velocity within a category. Used as a demand proxy: BULLIANT leather wallet BSR = 8,365 units/month.</t>
         </is>
       </c>
-      <c r="D14" s="97" t="inlineStr">
+      <c r="D14" s="95" t="inlineStr">
         <is>
           <t>Proxy Data</t>
         </is>
@@ -8995,7 +8935,7 @@
           <t>US regulatory body enforcing truthful product labeling. The FTC Guides for Textile &amp; Leather (MAT-001) require accurate leather grade disclosure.</t>
         </is>
       </c>
-      <c r="D15" s="98" t="inlineStr">
+      <c r="D15" s="96" t="inlineStr">
         <is>
           <t>PRD · OKRs · Impl. Map</t>
         </is>
@@ -9017,7 +8957,7 @@
           <t>The FTC guide prohibiting bonded, split, or PU leather from being labeled "genuine leather." Violation risk: product delisting + fines. The AI classifier enforces this at ingestion.</t>
         </is>
       </c>
-      <c r="D16" s="97" t="inlineStr">
+      <c r="D16" s="95" t="inlineStr">
         <is>
           <t>PRD · OKRs · Impl. Map</t>
         </is>
@@ -9039,7 +8979,7 @@
           <t>California law requiring businesses to warn consumers about significant exposures to chemicals causing cancer or reproductive harm. Chrome-tanned leather may trigger Prop 65 disclosure on Amazon.</t>
         </is>
       </c>
-      <c r="D17" s="98" t="inlineStr">
+      <c r="D17" s="96" t="inlineStr">
         <is>
           <t>Impl. Map · Roadmap</t>
         </is>
@@ -9061,7 +9001,7 @@
           <t>International certification body for environmentally responsible leather production. Grades: Gold / Silver / Bronze. Referenced in eco_claims schema field (V2 scope).</t>
         </is>
       </c>
-      <c r="D18" s="97" t="inlineStr">
+      <c r="D18" s="95" t="inlineStr">
         <is>
           <t>Impl. Map · References</t>
         </is>
@@ -9083,7 +9023,7 @@
           <t>International certification confirming leather/textiles are free from harmful substances. Relevant for eco_claims field and EU market compliance.</t>
         </is>
       </c>
-      <c r="D19" s="98" t="inlineStr">
+      <c r="D19" s="96" t="inlineStr">
         <is>
           <t>Impl. Map</t>
         </is>
@@ -9105,7 +9045,7 @@
           <t>EU regulation restricting hazardous substances in products. Relevant for chrome-tanned leather sold in EU — Cr(VI) limits apply.</t>
         </is>
       </c>
-      <c r="D20" s="97" t="inlineStr">
+      <c r="D20" s="95" t="inlineStr">
         <is>
           <t>Impl. Map</t>
         </is>
@@ -9127,7 +9067,7 @@
           <t>Amazon's API for marketplace integrations. Printify must apply for SP-API approval (~2–4 weeks) to list leather products with LeatherType node and Prop 65 auto-disclosure.</t>
         </is>
       </c>
-      <c r="D21" s="98" t="inlineStr">
+      <c r="D21" s="96" t="inlineStr">
         <is>
           <t>Roadmap · Impl. Map</t>
         </is>
@@ -9149,7 +9089,7 @@
           <t>Custom data fields extending Shopify product records beyond standard attributes. Printify uses these to pass material attributes (leather_grade, tanning_method) to Shopify channel. No indexing lag vs. Amazon.</t>
         </is>
       </c>
-      <c r="D22" s="97" t="inlineStr">
+      <c r="D22" s="95" t="inlineStr">
         <is>
           <t>Roadmap · PRD</t>
         </is>
@@ -9171,7 +9111,7 @@
           <t>Core material classification: full_grain / top_grain / corrected_grain / split / bonded / pu / vegan. Anchors FTC MAT-001 compliance and marketplace category routing.</t>
         </is>
       </c>
-      <c r="D23" s="98" t="inlineStr">
+      <c r="D23" s="96" t="inlineStr">
         <is>
           <t>PRD · Impl. Map</t>
         </is>
@@ -9193,7 +9133,7 @@
           <t>How the hide was treated: vegetable / chrome / chrome_free / combination. Chrome triggers Prop 65 auto-disclosure on Amazon.</t>
         </is>
       </c>
-      <c r="D24" s="97" t="inlineStr">
+      <c r="D24" s="95" t="inlineStr">
         <is>
           <t>PRD · Impl. Map</t>
         </is>
@@ -9215,7 +9155,7 @@
           <t>Boolean: true = corrected (sanded) grain surface, false = natural grain. Required to prevent misclassifying corrected top_grain as full_grain.</t>
         </is>
       </c>
-      <c r="D25" s="98" t="inlineStr">
+      <c r="D25" s="96" t="inlineStr">
         <is>
           <t>PRD · Impl. Map</t>
         </is>
@@ -9237,7 +9177,7 @@
           <t>Array enum: ftc_genuine / prop_65_ca / mat_001_approved / none. Drives listing gate logic — "none" blocks listing on Amazon channel.</t>
         </is>
       </c>
-      <c r="D26" s="97" t="inlineStr">
+      <c r="D26" s="95" t="inlineStr">
         <is>
           <t>PRD · Impl. Map</t>
         </is>
@@ -9259,7 +9199,7 @@
           <t>Array enum: lwg_gold / lwg_silver / oeko_tex / reach_compliant / none. MVP 2 scope — powers ECO badge on PDP and EU channel compliance.</t>
         </is>
       </c>
-      <c r="D27" s="98" t="inlineStr">
+      <c r="D27" s="96" t="inlineStr">
         <is>
           <t>PRD · Impl. Map</t>
         </is>
@@ -9281,7 +9221,7 @@
           <t>A predefined performance threshold that, if not met, triggers immediate halt of investment. This PRD's kill gate: &lt;15 orders/SKU at Month 2 post-launch → halt &amp; reallocate team.</t>
         </is>
       </c>
-      <c r="D28" s="97" t="inlineStr">
+      <c r="D28" s="95" t="inlineStr">
         <is>
           <t>Throughout</t>
         </is>
@@ -9303,7 +9243,7 @@
           <t>A structured decision point between project phases where continuation is contingent on meeting predefined criteria. Each phase must earn the right to spend the next budget tranche.</t>
         </is>
       </c>
-      <c r="D29" s="98" t="inlineStr">
+      <c r="D29" s="96" t="inlineStr">
         <is>
           <t>Throughout</t>
         </is>
@@ -9325,7 +9265,7 @@
           <t>A native AI agent that reads a supplier's product name + data sheet and pre-fills the 8 schema fields. Reduces form error rate from ~20–35% (unassisted) to &lt;10%.</t>
         </is>
       </c>
-      <c r="D30" s="97" t="inlineStr">
+      <c r="D30" s="95" t="inlineStr">
         <is>
           <t>PRD · OKRs</t>
         </is>

</xml_diff>